<commit_message>
fix: check mitochondria proteins
</commit_message>
<xml_diff>
--- a/data/sce_compartment_curation/mitochondrial_inner_membrane_annotations_manual_v3.xlsx
+++ b/data/sce_compartment_curation/mitochondrial_inner_membrane_annotations_manual_v3.xlsx
@@ -441,7 +441,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>YOR266W</t>
+          <t>YDR032C</t>
         </is>
       </c>
     </row>
@@ -451,7 +451,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>YOL059W</t>
+          <t>YBR039W</t>
         </is>
       </c>
     </row>
@@ -461,7 +461,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>YDR393W</t>
+          <t>YPR116W</t>
         </is>
       </c>
     </row>
@@ -471,7 +471,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>YPL109C</t>
+          <t>YEL030W</t>
         </is>
       </c>
     </row>
@@ -481,7 +481,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>YLR067C</t>
+          <t>YNR017W</t>
         </is>
       </c>
     </row>
@@ -491,7 +491,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>YML081C-A</t>
+          <t>YGL129C</t>
         </is>
       </c>
     </row>
@@ -501,7 +501,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>YEL020W-A</t>
+          <t>YBR084W</t>
         </is>
       </c>
     </row>
@@ -511,7 +511,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>YNL100W</t>
+          <t>YFR011C</t>
         </is>
       </c>
     </row>
@@ -521,7 +521,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>YJL054W</t>
+          <t>YJL003W</t>
         </is>
       </c>
     </row>
@@ -531,7 +531,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>YHR002W</t>
+          <t>YER166W</t>
         </is>
       </c>
     </row>
@@ -541,7 +541,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>YBR291C</t>
+          <t>YOR086C</t>
         </is>
       </c>
     </row>
@@ -551,7 +551,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>YGR183C</t>
+          <t>YOR334W</t>
         </is>
       </c>
     </row>
@@ -561,7 +561,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>YMR024W</t>
+          <t>YMR256C</t>
         </is>
       </c>
     </row>
@@ -571,7 +571,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>YDL164C</t>
+          <t>YOL008W</t>
         </is>
       </c>
     </row>
@@ -581,7 +581,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>YDR381C-A</t>
+          <t>YDR237W</t>
         </is>
       </c>
     </row>
@@ -591,7 +591,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>YJL062W-A</t>
+          <t>YDL142C</t>
         </is>
       </c>
     </row>
@@ -601,7 +601,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>YKL016C</t>
+          <t>YDR282C</t>
         </is>
       </c>
     </row>
@@ -611,7 +611,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>YDL085W</t>
+          <t>YMR177W</t>
         </is>
       </c>
     </row>
@@ -621,7 +621,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>YMR023C</t>
+          <t>YIL077C</t>
         </is>
       </c>
     </row>
@@ -631,7 +631,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>YMR212C</t>
+          <t>YMR150C</t>
         </is>
       </c>
     </row>
@@ -641,7 +641,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>YOR334W</t>
+          <t>YNL177C</t>
         </is>
       </c>
     </row>
@@ -651,7 +651,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>YHR162W</t>
+          <t>YGR147C</t>
         </is>
       </c>
     </row>
@@ -661,7 +661,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>YBL095W</t>
+          <t>YCL017C</t>
         </is>
       </c>
     </row>
@@ -671,7 +671,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>YIL157C</t>
+          <t>YMR188C</t>
         </is>
       </c>
     </row>
@@ -681,7 +681,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Q0275</t>
+          <t>YPL168W</t>
         </is>
       </c>
     </row>
@@ -691,7 +691,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>YDL215C</t>
+          <t>YPL078C</t>
         </is>
       </c>
     </row>
@@ -701,7 +701,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>YOR176W</t>
+          <t>Q0070</t>
         </is>
       </c>
     </row>
@@ -711,7 +711,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>YDR298C</t>
+          <t>Q0250</t>
         </is>
       </c>
     </row>
@@ -721,7 +721,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>YBR078W</t>
+          <t>YHR198C</t>
         </is>
       </c>
     </row>
@@ -731,7 +731,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>YHR199C</t>
+          <t>YNL122C</t>
         </is>
       </c>
     </row>
@@ -741,7 +741,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>YLR090W</t>
+          <t>YKR042W</t>
         </is>
       </c>
     </row>
@@ -751,7 +751,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>YMR177W</t>
+          <t>YMR302C</t>
         </is>
       </c>
     </row>
@@ -761,7 +761,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>YNL315C</t>
+          <t>YHR168W</t>
         </is>
       </c>
     </row>
@@ -771,7 +771,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>YOR350C</t>
+          <t>YJR003C</t>
         </is>
       </c>
     </row>
@@ -781,7 +781,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>YLR290C</t>
+          <t>YNR002C</t>
         </is>
       </c>
     </row>
@@ -791,7 +791,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Q0105</t>
+          <t>YJL143W</t>
         </is>
       </c>
     </row>
@@ -801,7 +801,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>YJR095W</t>
+          <t>YDR204W</t>
         </is>
       </c>
     </row>
@@ -811,7 +811,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>YMR150C</t>
+          <t>YML120C</t>
         </is>
       </c>
     </row>
@@ -821,7 +821,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>YMR089C</t>
+          <t>YDR298C</t>
         </is>
       </c>
     </row>
@@ -831,7 +831,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>YPR033C</t>
+          <t>YDL174C</t>
         </is>
       </c>
     </row>
@@ -841,7 +841,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>YJL171C</t>
+          <t>YKL106W</t>
         </is>
       </c>
     </row>
@@ -851,7 +851,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>YGR174C</t>
+          <t>YBR003W</t>
         </is>
       </c>
     </row>
@@ -861,7 +861,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>YNL005C</t>
+          <t>YBR044C</t>
         </is>
       </c>
     </row>
@@ -871,7 +871,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Q0140</t>
+          <t>YPR149W</t>
         </is>
       </c>
     </row>
@@ -881,7 +881,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>YOR232W</t>
+          <t>YMR228W</t>
         </is>
       </c>
     </row>
@@ -891,7 +891,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>YGL057C</t>
+          <t>YDR462W</t>
         </is>
       </c>
     </row>
@@ -901,7 +901,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Q0070</t>
+          <t>YER053C</t>
         </is>
       </c>
     </row>
@@ -911,7 +911,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>YBR024W</t>
+          <t>YER077C</t>
         </is>
       </c>
     </row>
@@ -921,7 +921,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>YDR405W</t>
+          <t>YOL027C</t>
         </is>
       </c>
     </row>
@@ -931,7 +931,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>YGL191W</t>
+          <t>YNL185C</t>
         </is>
       </c>
     </row>
@@ -941,7 +941,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>YJL063C</t>
+          <t>YIR021W</t>
         </is>
       </c>
     </row>
@@ -951,7 +951,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>YPL215W</t>
+          <t>YKL195W</t>
         </is>
       </c>
     </row>
@@ -961,7 +961,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>YDL183C</t>
+          <t>YMR212C</t>
         </is>
       </c>
     </row>
@@ -971,7 +971,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>YML072C</t>
+          <t>YOR022C</t>
         </is>
       </c>
     </row>
@@ -981,7 +981,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>YER020W</t>
+          <t>YHR005C-A</t>
         </is>
       </c>
     </row>
@@ -991,7 +991,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>YKL162C</t>
+          <t>YHL014C</t>
         </is>
       </c>
     </row>
@@ -1001,7 +1001,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>YOR037W</t>
+          <t>YOR211C</t>
         </is>
       </c>
     </row>
@@ -1011,7 +1011,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>YMR003W</t>
+          <t>YJL161W</t>
         </is>
       </c>
     </row>
@@ -1021,7 +1021,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>YIL134W</t>
+          <t>YMR241W</t>
         </is>
       </c>
     </row>
@@ -1031,7 +1031,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>YDR347W</t>
+          <t>YKL087C</t>
         </is>
       </c>
     </row>
@@ -1041,7 +1041,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>YBR121C</t>
+          <t>YMR193W</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>YFR033C</t>
+          <t>YDR347W</t>
         </is>
       </c>
     </row>
@@ -1061,7 +1061,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>YBR262C</t>
+          <t>YOL095C</t>
         </is>
       </c>
     </row>
@@ -1071,7 +1071,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Q0085</t>
+          <t>YPL029W</t>
         </is>
       </c>
     </row>
@@ -1081,7 +1081,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Q0250</t>
+          <t>YFL016C</t>
         </is>
       </c>
     </row>
@@ -1091,7 +1091,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>YJL045W</t>
+          <t>YLR239C</t>
         </is>
       </c>
     </row>
@@ -1101,7 +1101,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>YGR193C</t>
+          <t>YIL022W</t>
         </is>
       </c>
     </row>
@@ -1111,7 +1111,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>YNL256W</t>
+          <t>YBR227C</t>
         </is>
       </c>
     </row>
@@ -1121,7 +1121,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>YIL111W</t>
+          <t>YBR078W</t>
         </is>
       </c>
     </row>
@@ -1131,7 +1131,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Q0130</t>
+          <t>YNR040W</t>
         </is>
       </c>
     </row>
@@ -1141,7 +1141,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>YPL005W</t>
+          <t>YKL133C</t>
         </is>
       </c>
     </row>
@@ -1151,7 +1151,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>YDR185C</t>
+          <t>YDR079W</t>
         </is>
       </c>
     </row>
@@ -1161,7 +1161,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>YKL208W</t>
+          <t>YGR174C</t>
         </is>
       </c>
     </row>
@@ -1171,7 +1171,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Q0110</t>
+          <t>YGR096W</t>
         </is>
       </c>
     </row>
@@ -1181,7 +1181,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>YDR316W</t>
+          <t>YGR236C</t>
         </is>
       </c>
     </row>
@@ -1191,7 +1191,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>YBL013W</t>
+          <t>YHR120W</t>
         </is>
       </c>
     </row>
@@ -1201,7 +1201,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>YKR052C</t>
+          <t>YNL100W</t>
         </is>
       </c>
     </row>
@@ -1211,7 +1211,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>YOR205C</t>
+          <t>YPL060W</t>
         </is>
       </c>
     </row>
@@ -1221,7 +1221,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>YML128C</t>
+          <t>YNL306W</t>
         </is>
       </c>
     </row>
@@ -1231,7 +1231,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>YFR011C</t>
+          <t>YER153C</t>
         </is>
       </c>
     </row>
@@ -1241,7 +1241,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>YPL060W</t>
+          <t>YMR066W</t>
         </is>
       </c>
     </row>
@@ -1251,7 +1251,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>YPR020W</t>
+          <t>YGL136C</t>
         </is>
       </c>
     </row>
@@ -1261,7 +1261,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>YIL155C</t>
+          <t>YJL147C</t>
         </is>
       </c>
     </row>
@@ -1271,7 +1271,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Q0055</t>
+          <t>YJR045C</t>
         </is>
       </c>
     </row>
@@ -1281,7 +1281,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>YMR066W</t>
+          <t>YLR342W</t>
         </is>
       </c>
     </row>
@@ -1291,7 +1291,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>YMR256C</t>
+          <t>YBR192W</t>
         </is>
       </c>
     </row>
@@ -1301,7 +1301,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>YPL029W</t>
+          <t>YDR258C</t>
         </is>
       </c>
     </row>
@@ -1311,7 +1311,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>YMR097C</t>
+          <t>YLR251W</t>
         </is>
       </c>
     </row>
@@ -1321,7 +1321,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>YJL143W</t>
+          <t>YGR222W</t>
         </is>
       </c>
     </row>
@@ -1331,7 +1331,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>YNL137C</t>
+          <t>YCL057C-A</t>
         </is>
       </c>
     </row>
@@ -1341,7 +1341,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>YKL148C</t>
+          <t>YGR046W</t>
         </is>
       </c>
     </row>
@@ -1351,7 +1351,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Q0080</t>
+          <t>YBR104W</t>
         </is>
       </c>
     </row>
@@ -1361,7 +1361,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>YBR054W</t>
+          <t>YER020W</t>
         </is>
       </c>
     </row>
@@ -1371,7 +1371,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>YDR233C</t>
+          <t>YOR201C</t>
         </is>
       </c>
     </row>
@@ -1381,7 +1381,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>YNL009W</t>
+          <t>YDR375C</t>
         </is>
       </c>
     </row>
@@ -1391,7 +1391,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>YKR065C</t>
+          <t>YJL102W</t>
         </is>
       </c>
     </row>
@@ -1401,7 +1401,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>YMR193W</t>
+          <t>YMR024W</t>
         </is>
       </c>
     </row>
@@ -1411,7 +1411,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>YNR041C</t>
+          <t>YIL157C</t>
         </is>
       </c>
     </row>
@@ -1421,7 +1421,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>YBL030C</t>
+          <t>YNL071W</t>
         </is>
       </c>
     </row>
@@ -1431,7 +1431,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>YDL142C</t>
+          <t>YLR188W</t>
         </is>
       </c>
     </row>
@@ -1441,7 +1441,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>YNL211C</t>
+          <t>YPL222W</t>
         </is>
       </c>
     </row>
@@ -1451,7 +1451,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>YLR439W</t>
+          <t>YOR221C</t>
         </is>
       </c>
     </row>
@@ -1461,7 +1461,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>YDR116C</t>
+          <t>YDL222C</t>
         </is>
       </c>
     </row>
@@ -1471,7 +1471,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>YDL027C</t>
+          <t>YBR163W</t>
         </is>
       </c>
     </row>
@@ -1481,7 +1481,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>YLR348C</t>
+          <t>YJL023C</t>
         </is>
       </c>
     </row>
@@ -1491,7 +1491,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>YNL185C</t>
+          <t>YKL148C</t>
         </is>
       </c>
     </row>
@@ -1501,7 +1501,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>YCL009C</t>
+          <t>YOR305W</t>
         </is>
       </c>
     </row>
@@ -1511,7 +1511,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>YNR002C</t>
+          <t>Q0130</t>
         </is>
       </c>
     </row>
@@ -1521,7 +1521,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>YGR171C</t>
+          <t>YDR322C-A</t>
         </is>
       </c>
     </row>
@@ -1531,7 +1531,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>YDR375C</t>
+          <t>YHR194W</t>
         </is>
       </c>
     </row>
@@ -1541,7 +1541,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>YBL038W</t>
+          <t>YOR017W</t>
         </is>
       </c>
     </row>
@@ -1551,7 +1551,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>YPR125W</t>
+          <t>YKL217W</t>
         </is>
       </c>
     </row>
@@ -1561,7 +1561,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>YPL172C</t>
+          <t>YLR253W</t>
         </is>
       </c>
     </row>
@@ -1571,7 +1571,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>YDL222C</t>
+          <t>YNL125C</t>
         </is>
       </c>
     </row>
@@ -1581,7 +1581,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>YPL063W</t>
+          <t>YGR165W</t>
         </is>
       </c>
     </row>
@@ -1591,7 +1591,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>YKL056C</t>
+          <t>Q0140</t>
         </is>
       </c>
     </row>
@@ -1601,7 +1601,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>YLR203C</t>
+          <t>YJR121W</t>
         </is>
       </c>
     </row>
@@ -1611,7 +1611,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>YKL120W</t>
+          <t>YGL107C</t>
         </is>
       </c>
     </row>
@@ -1621,7 +1621,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>YDR258C</t>
+          <t>YDR185C</t>
         </is>
       </c>
     </row>
@@ -1631,7 +1631,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>YBR084W</t>
+          <t>YGR235C</t>
         </is>
       </c>
     </row>
@@ -1641,7 +1641,7 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>YGR235C</t>
+          <t>YPL097W</t>
         </is>
       </c>
     </row>
@@ -1651,7 +1651,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>YLR059C</t>
+          <t>YNL009W</t>
         </is>
       </c>
     </row>
@@ -1661,7 +1661,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>YOR100C</t>
+          <t>YGR116W</t>
         </is>
       </c>
     </row>
@@ -1671,7 +1671,7 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>YNL177C</t>
+          <t>YJR077C</t>
         </is>
       </c>
     </row>
@@ -1681,7 +1681,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>YLR188W</t>
+          <t>YEL024W</t>
         </is>
       </c>
     </row>
@@ -1691,7 +1691,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>YPL099C</t>
+          <t>YDL164C</t>
         </is>
       </c>
     </row>
@@ -1701,7 +1701,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>YKL170W</t>
+          <t>YLR084C</t>
         </is>
       </c>
     </row>
@@ -1711,7 +1711,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>YDR119W-A</t>
+          <t>YGR062C</t>
         </is>
       </c>
     </row>
@@ -1721,7 +1721,7 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>YOR211C</t>
+          <t>YPR191W</t>
         </is>
       </c>
     </row>
@@ -1731,7 +1731,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>YGR062C</t>
+          <t>YPL224C</t>
         </is>
       </c>
     </row>
@@ -1741,7 +1741,7 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>YGL226W</t>
+          <t>YDR322W</t>
         </is>
       </c>
     </row>
@@ -1751,7 +1751,7 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>YLR312W-A</t>
+          <t>YPR024W</t>
         </is>
       </c>
     </row>
@@ -1761,7 +1761,7 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>YDL067C</t>
+          <t>YNL256W</t>
         </is>
       </c>
     </row>
@@ -1771,7 +1771,7 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>YIR024C</t>
+          <t>YIL111W</t>
         </is>
       </c>
     </row>
@@ -1781,7 +1781,7 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>YMR166C</t>
+          <t>YBL045C</t>
         </is>
       </c>
     </row>
@@ -1791,7 +1791,7 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>YBL059W</t>
+          <t>YDR494W</t>
         </is>
       </c>
     </row>
@@ -1801,7 +1801,7 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>Q0045</t>
+          <t>YJL180C</t>
         </is>
       </c>
     </row>
@@ -1811,7 +1811,7 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>YGR084C</t>
+          <t>YDR393W</t>
         </is>
       </c>
     </row>
@@ -1821,7 +1821,7 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>YPR166C</t>
+          <t>YJL104W</t>
         </is>
       </c>
     </row>
@@ -1831,7 +1831,7 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>YDR384C</t>
+          <t>YNR018W</t>
         </is>
       </c>
     </row>
@@ -1841,7 +1841,7 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>YKL138C</t>
+          <t>YOR297C</t>
         </is>
       </c>
     </row>
@@ -1851,7 +1851,7 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>YDL207W</t>
+          <t>YLR290C</t>
         </is>
       </c>
     </row>
@@ -1861,7 +1861,7 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>YOL077W-A</t>
+          <t>YDR116C</t>
         </is>
       </c>
     </row>
@@ -1871,7 +1871,7 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>YFR045W</t>
+          <t>YOR354C</t>
         </is>
       </c>
     </row>
@@ -1881,7 +1881,7 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>YEL006W</t>
+          <t>YKR052C</t>
         </is>
       </c>
     </row>
@@ -1891,7 +1891,7 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>YDR282C</t>
+          <t>YBL059W</t>
         </is>
       </c>
     </row>
@@ -1901,7 +1901,7 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>YMR157C</t>
+          <t>YHR147C</t>
         </is>
       </c>
     </row>
@@ -1911,7 +1911,7 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>YDR041W</t>
+          <t>YPL005W</t>
         </is>
       </c>
     </row>
@@ -1921,7 +1921,7 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>YIL016W</t>
+          <t>YML128C</t>
         </is>
       </c>
     </row>
@@ -1931,7 +1931,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>YGR096W</t>
+          <t>YEL059C-A</t>
         </is>
       </c>
     </row>
@@ -1941,7 +1941,7 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>YJR045C</t>
+          <t>YMR158W</t>
         </is>
       </c>
     </row>
@@ -1951,7 +1951,7 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>YBR227C</t>
+          <t>YKL055C</t>
         </is>
       </c>
     </row>
@@ -1961,7 +1961,7 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>YER086W</t>
+          <t>YDR350C</t>
         </is>
       </c>
     </row>
@@ -1971,7 +1971,7 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>YOR065W</t>
+          <t>YPL134C</t>
         </is>
       </c>
     </row>
@@ -1981,7 +1981,7 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>YJR080C</t>
+          <t>YER069W</t>
         </is>
       </c>
     </row>
@@ -1991,7 +1991,7 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>YPR021C</t>
+          <t>YBR282W</t>
         </is>
       </c>
     </row>
@@ -2001,7 +2001,7 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>YER154W</t>
+          <t>YDR194C</t>
         </is>
       </c>
     </row>
@@ -2011,7 +2011,7 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>YML025C</t>
+          <t>YLR312W-A</t>
         </is>
       </c>
     </row>
@@ -2021,7 +2021,7 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>YEL052W</t>
+          <t>YBL038W</t>
         </is>
       </c>
     </row>
@@ -2031,7 +2031,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>YHL004W</t>
+          <t>YKL155C</t>
         </is>
       </c>
     </row>
@@ -2041,7 +2041,7 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>YCR004C</t>
+          <t>YPL215W</t>
         </is>
       </c>
     </row>
@@ -2051,7 +2051,7 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>YJL180C</t>
+          <t>YOL053W</t>
         </is>
       </c>
     </row>
@@ -2061,7 +2061,7 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>YDR032C</t>
+          <t>YGL191W</t>
         </is>
       </c>
     </row>
@@ -2071,7 +2071,7 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>YML129C</t>
+          <t>YMR108W</t>
         </is>
       </c>
     </row>
@@ -2081,7 +2081,7 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>YGL119W</t>
+          <t>YCL004W</t>
         </is>
       </c>
     </row>
@@ -2091,7 +2091,7 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>YBL045C</t>
+          <t>YGR084C</t>
         </is>
       </c>
     </row>
@@ -2101,7 +2101,7 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>YBR185C</t>
+          <t>YGR150C</t>
         </is>
       </c>
     </row>
@@ -2111,7 +2111,7 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>YOL042W</t>
+          <t>Q0105</t>
         </is>
       </c>
     </row>
@@ -2121,7 +2121,7 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>YGL136C</t>
+          <t>YOR196C</t>
         </is>
       </c>
     </row>
@@ -2131,7 +2131,7 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>YDR322W</t>
+          <t>YJR034W</t>
         </is>
       </c>
     </row>
@@ -2141,7 +2141,7 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>YLR139C</t>
+          <t>YGR110W</t>
         </is>
       </c>
     </row>
@@ -2151,7 +2151,7 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>YGL059W</t>
+          <t>YOR037W</t>
         </is>
       </c>
     </row>
@@ -2161,7 +2161,7 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>YKL087C</t>
+          <t>YHL004W</t>
         </is>
       </c>
     </row>
@@ -2171,7 +2171,7 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>YDL202W</t>
+          <t>YPL099C</t>
         </is>
       </c>
     </row>
@@ -2181,7 +2181,7 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>YOL023W</t>
+          <t>YOL077W-A</t>
         </is>
       </c>
     </row>
@@ -2191,7 +2191,7 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>YOR221C</t>
+          <t>YER182W</t>
         </is>
       </c>
     </row>
@@ -2201,7 +2201,7 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>YDR376W</t>
+          <t>YLR139C</t>
         </is>
       </c>
     </row>
@@ -2211,7 +2211,7 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>YER069W</t>
+          <t>YNL211C</t>
         </is>
       </c>
     </row>
@@ -2221,7 +2221,7 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>YER080W</t>
+          <t>YJL209W</t>
         </is>
       </c>
     </row>
@@ -2231,7 +2231,7 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>YER125W</t>
+          <t>YDL215C</t>
         </is>
       </c>
     </row>
@@ -2241,7 +2241,7 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>YEL059C-A</t>
+          <t>YGR171C</t>
         </is>
       </c>
     </row>
@@ -2251,7 +2251,7 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>YIL077C</t>
+          <t>YPR061C</t>
         </is>
       </c>
     </row>
@@ -2261,7 +2261,7 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>YJL104W</t>
+          <t>Q0110</t>
         </is>
       </c>
     </row>
@@ -2271,7 +2271,7 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>YOR022C</t>
+          <t>YOR125C</t>
         </is>
       </c>
     </row>
@@ -2281,7 +2281,7 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>YLL041C</t>
+          <t>YML072C</t>
         </is>
       </c>
     </row>
@@ -2291,7 +2291,7 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>YBR085W</t>
+          <t>YLR395C</t>
         </is>
       </c>
     </row>
@@ -2301,7 +2301,7 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>YJR003C</t>
+          <t>YGL057C</t>
         </is>
       </c>
     </row>
@@ -2311,7 +2311,7 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>YBR047W</t>
+          <t>YMR038C</t>
         </is>
       </c>
     </row>
@@ -2331,7 +2331,7 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>YER166W</t>
+          <t>YMR023C</t>
         </is>
       </c>
     </row>
@@ -2341,7 +2341,7 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>YGR150C</t>
+          <t>YLR164W</t>
         </is>
       </c>
     </row>
@@ -2351,7 +2351,7 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>YOL053W</t>
+          <t>YMR003W</t>
         </is>
       </c>
     </row>
@@ -2361,7 +2361,7 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>YMR257C</t>
+          <t>YOL096C</t>
         </is>
       </c>
     </row>
@@ -2371,7 +2371,7 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>YKL155C</t>
+          <t>YKR016W</t>
         </is>
       </c>
     </row>
@@ -2381,7 +2381,7 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>YER168C</t>
+          <t>YBR185C</t>
         </is>
       </c>
     </row>
@@ -2391,7 +2391,7 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>YPR149W</t>
+          <t>YNL169C</t>
         </is>
       </c>
     </row>
@@ -2401,7 +2401,7 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>YLR239C</t>
+          <t>YER183C</t>
         </is>
       </c>
     </row>
@@ -2411,7 +2411,7 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>YMR098C</t>
+          <t>YFR033C</t>
         </is>
       </c>
     </row>
@@ -2421,7 +2421,7 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>YHR005C-A</t>
+          <t>YLR390W</t>
         </is>
       </c>
     </row>
@@ -2431,7 +2431,7 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>YHR120W</t>
+          <t>YBR091C</t>
         </is>
       </c>
     </row>
@@ -2441,7 +2441,7 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>YMR056C</t>
+          <t>YKL162C</t>
         </is>
       </c>
     </row>
@@ -2451,7 +2451,7 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>YHR147C</t>
+          <t>YLR203C</t>
         </is>
       </c>
     </row>
@@ -2461,7 +2461,7 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>YLR084C</t>
+          <t>YDL067C</t>
         </is>
       </c>
     </row>
@@ -2471,7 +2471,7 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>YBR003W</t>
+          <t>YBR251W</t>
         </is>
       </c>
     </row>
@@ -2481,7 +2481,7 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>YJL102W</t>
+          <t>YPL172C</t>
         </is>
       </c>
     </row>
@@ -2491,7 +2491,7 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>YOL008W</t>
+          <t>YOR176W</t>
         </is>
       </c>
     </row>
@@ -2501,7 +2501,7 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>YJR101W</t>
+          <t>YPL063W</t>
         </is>
       </c>
     </row>
@@ -2511,7 +2511,7 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>YJR034W</t>
+          <t>Q0045</t>
         </is>
       </c>
     </row>
@@ -2521,7 +2521,7 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>YFL016C</t>
+          <t>YGL059W</t>
         </is>
       </c>
     </row>
@@ -2531,7 +2531,7 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>YBR037C</t>
+          <t>YKL029C</t>
         </is>
       </c>
     </row>
@@ -2541,7 +2541,7 @@
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>YJL003W</t>
+          <t>YGR193C</t>
         </is>
       </c>
     </row>
@@ -2551,7 +2551,7 @@
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>YOL095C</t>
+          <t>YEL052W</t>
         </is>
       </c>
     </row>
@@ -2561,7 +2561,7 @@
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>YOL096C</t>
+          <t>YOL023W</t>
         </is>
       </c>
     </row>
@@ -2571,7 +2571,7 @@
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>Q0050</t>
+          <t>YIL105C</t>
         </is>
       </c>
     </row>
@@ -2581,7 +2581,7 @@
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>YDL036C</t>
+          <t>YDL069C</t>
         </is>
       </c>
     </row>
@@ -2591,7 +2591,7 @@
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>YLR382C</t>
+          <t>YMR089C</t>
         </is>
       </c>
     </row>
@@ -2601,7 +2601,7 @@
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>YER017C</t>
+          <t>YAL039C</t>
         </is>
       </c>
     </row>
@@ -2611,7 +2611,7 @@
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>Q0120</t>
+          <t>YLR201C</t>
         </is>
       </c>
     </row>
@@ -2621,7 +2621,7 @@
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>YDR058C</t>
+          <t>YLR289W</t>
         </is>
       </c>
     </row>
@@ -2631,7 +2631,7 @@
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>YGL080W</t>
+          <t>YBR024W</t>
         </is>
       </c>
     </row>
@@ -2641,7 +2641,7 @@
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>YLR201C</t>
+          <t>YDR384C</t>
         </is>
       </c>
     </row>
@@ -2651,7 +2651,7 @@
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>YAL054C</t>
+          <t>Q0085</t>
         </is>
       </c>
     </row>
@@ -2661,7 +2661,7 @@
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>YOR086C</t>
+          <t>YNL052W</t>
         </is>
       </c>
     </row>
@@ -2671,7 +2671,7 @@
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>YHR001W-A</t>
+          <t>YNL328C</t>
         </is>
       </c>
     </row>
@@ -2681,7 +2681,7 @@
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>YNL169C</t>
+          <t>YGR112W</t>
         </is>
       </c>
     </row>
@@ -2691,7 +2691,7 @@
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>YCR010C</t>
+          <t>YPL103C</t>
         </is>
       </c>
     </row>
@@ -2701,7 +2701,7 @@
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>YHR011W</t>
+          <t>YNL137C</t>
         </is>
       </c>
     </row>
@@ -2711,7 +2711,7 @@
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>YLR395C</t>
+          <t>YJR080C</t>
         </is>
       </c>
     </row>
@@ -2721,7 +2721,7 @@
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>YDR231C</t>
+          <t>YER019W</t>
         </is>
       </c>
     </row>
@@ -2731,7 +2731,7 @@
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>YJL166W</t>
+          <t>YDR232W</t>
         </is>
       </c>
     </row>
@@ -2741,7 +2741,7 @@
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>YBL022C</t>
+          <t>YDR119W-A</t>
         </is>
       </c>
     </row>
@@ -2751,7 +2751,7 @@
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>YBR282W</t>
+          <t>YIR024C</t>
         </is>
       </c>
     </row>
@@ -2761,7 +2761,7 @@
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>YGR257C</t>
+          <t>YBR037C</t>
         </is>
       </c>
     </row>
@@ -2771,7 +2771,7 @@
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>YPL103C</t>
+          <t>YJL208C</t>
         </is>
       </c>
     </row>
@@ -2781,7 +2781,7 @@
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>YDL004W</t>
+          <t>YLR193C</t>
         </is>
       </c>
     </row>
@@ -2791,7 +2791,7 @@
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>YKL187C</t>
+          <t>YMR282C</t>
         </is>
       </c>
     </row>
@@ -2801,7 +2801,7 @@
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>YMR241W</t>
+          <t>YBL099W</t>
         </is>
       </c>
     </row>
@@ -2811,7 +2811,7 @@
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>YNL122C</t>
+          <t>YDL027C</t>
         </is>
       </c>
     </row>
@@ -2821,7 +2821,7 @@
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>YER019W</t>
+          <t>YIL042C</t>
         </is>
       </c>
     </row>
@@ -2831,7 +2831,7 @@
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>YMR302C</t>
+          <t>YMR157C</t>
         </is>
       </c>
     </row>
@@ -2841,7 +2841,7 @@
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>YGR112W</t>
+          <t>YLR077W</t>
         </is>
       </c>
     </row>
@@ -2851,7 +2851,7 @@
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>YGR236C</t>
+          <t>YDL004W</t>
         </is>
       </c>
     </row>
@@ -2861,7 +2861,7 @@
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>YNL052W</t>
+          <t>YMR064W</t>
         </is>
       </c>
     </row>
@@ -2871,7 +2871,7 @@
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>YML091C</t>
+          <t>YDL036C</t>
         </is>
       </c>
     </row>
@@ -2881,7 +2881,7 @@
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>YBR163W</t>
+          <t>YPR020W</t>
         </is>
       </c>
     </row>
@@ -2891,7 +2891,7 @@
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>YNL252C</t>
+          <t>YBR291C</t>
         </is>
       </c>
     </row>
@@ -2901,7 +2901,7 @@
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>YDR065W</t>
+          <t>YHR011W</t>
         </is>
       </c>
     </row>
@@ -2911,7 +2911,7 @@
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>YJL161W</t>
+          <t>YGR255C</t>
         </is>
       </c>
     </row>
@@ -2921,7 +2921,7 @@
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>YLR008C</t>
+          <t>YMR115W</t>
         </is>
       </c>
     </row>
@@ -2931,7 +2931,7 @@
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>YHR198C</t>
+          <t>YGL226W</t>
         </is>
       </c>
     </row>
@@ -2941,7 +2941,7 @@
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>YKL011C</t>
+          <t>YER086W</t>
         </is>
       </c>
     </row>
@@ -2951,7 +2951,7 @@
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>YJL208C</t>
+          <t>YJR100C</t>
         </is>
       </c>
     </row>
@@ -2961,7 +2961,7 @@
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>YER183C</t>
+          <t>YKL003C</t>
         </is>
       </c>
     </row>
@@ -2971,7 +2971,7 @@
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>YGL236C</t>
+          <t>YLR382C</t>
         </is>
       </c>
     </row>
@@ -2981,7 +2981,7 @@
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>YMR282C</t>
+          <t>YEL006W</t>
         </is>
       </c>
     </row>
@@ -2991,7 +2991,7 @@
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>YNL328C</t>
+          <t>YNL315C</t>
         </is>
       </c>
     </row>
@@ -3001,7 +3001,7 @@
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>YOR354C</t>
+          <t>YGR033C</t>
         </is>
       </c>
     </row>
@@ -3011,7 +3011,7 @@
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>YHR100C</t>
+          <t>YNL252C</t>
         </is>
       </c>
     </row>
@@ -3021,7 +3021,7 @@
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>YLR164W</t>
+          <t>YDL202W</t>
         </is>
       </c>
     </row>
@@ -3031,7 +3031,7 @@
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>YGR116W</t>
+          <t>YFR045W</t>
         </is>
       </c>
     </row>
@@ -3041,7 +3041,7 @@
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>YGR110W</t>
+          <t>YDR033W</t>
         </is>
       </c>
     </row>
@@ -3051,7 +3051,7 @@
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>YKL055C</t>
+          <t>YJL062W-A</t>
         </is>
       </c>
     </row>
@@ -3061,7 +3061,7 @@
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>YER170W</t>
+          <t>YIL087C</t>
         </is>
       </c>
     </row>
@@ -3071,7 +3071,7 @@
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>YPL078C</t>
+          <t>YBL013W</t>
         </is>
       </c>
     </row>
@@ -3081,7 +3081,7 @@
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>YJL209W</t>
+          <t>YHR162W</t>
         </is>
       </c>
     </row>
@@ -3091,7 +3091,7 @@
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>YPL222W</t>
+          <t>YMR257C</t>
         </is>
       </c>
     </row>
@@ -3101,7 +3101,7 @@
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>YOR201C</t>
+          <t>YDL207W</t>
         </is>
       </c>
     </row>
@@ -3111,7 +3111,7 @@
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>YNL003C</t>
+          <t>YKL208W</t>
         </is>
       </c>
     </row>
@@ -3121,7 +3121,7 @@
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>YML110C</t>
+          <t>YJR095W</t>
         </is>
       </c>
     </row>
@@ -3131,7 +3131,7 @@
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>YDR197W</t>
+          <t>YHR002W</t>
         </is>
       </c>
     </row>
@@ -3141,7 +3141,7 @@
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>YER053C</t>
+          <t>YDR377W</t>
         </is>
       </c>
     </row>
@@ -3151,7 +3151,7 @@
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>YGR220C</t>
+          <t>YJL054W</t>
         </is>
       </c>
     </row>
@@ -3161,7 +3161,7 @@
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>YNR040W</t>
+          <t>YBL095W</t>
         </is>
       </c>
     </row>
@@ -3171,7 +3171,7 @@
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>YIL042C</t>
+          <t>YLR090W</t>
         </is>
       </c>
     </row>
@@ -3181,7 +3181,7 @@
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>YOR297C</t>
+          <t>YEL020W-A</t>
         </is>
       </c>
     </row>
@@ -3191,7 +3191,7 @@
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>YER182W</t>
+          <t>YOR330C</t>
         </is>
       </c>
     </row>
@@ -3201,7 +3201,7 @@
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>YPR061C</t>
+          <t>YKL138C</t>
         </is>
       </c>
     </row>
@@ -3211,7 +3211,7 @@
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>YER058W</t>
+          <t>YMR166C</t>
         </is>
       </c>
     </row>
@@ -3221,7 +3221,7 @@
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>YOR271C</t>
+          <t>YER058W</t>
         </is>
       </c>
     </row>
@@ -3231,7 +3231,7 @@
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>YJR100C</t>
+          <t>YIL016W</t>
         </is>
       </c>
     </row>
@@ -3241,7 +3241,7 @@
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>YOR147W</t>
+          <t>Q0050</t>
         </is>
       </c>
     </row>
@@ -3251,7 +3251,7 @@
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>YPL097W</t>
+          <t>YMR056C</t>
         </is>
       </c>
     </row>
@@ -3261,7 +3261,7 @@
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>YGR231C</t>
+          <t>YCR046C</t>
         </is>
       </c>
     </row>
@@ -3271,7 +3271,7 @@
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>YKR042W</t>
+          <t>YAL054C</t>
         </is>
       </c>
     </row>
@@ -3281,7 +3281,7 @@
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>YHR168W</t>
+          <t>YPL118W</t>
         </is>
       </c>
     </row>
@@ -3291,7 +3291,7 @@
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>YOR222W</t>
+          <t>YPR125W</t>
         </is>
       </c>
     </row>
@@ -3301,7 +3301,7 @@
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>YDR204W</t>
+          <t>YLL041C</t>
         </is>
       </c>
     </row>
@@ -3311,7 +3311,7 @@
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>YPL168W</t>
+          <t>YIL154C</t>
         </is>
       </c>
     </row>
@@ -3321,7 +3321,7 @@
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>YNR045W</t>
+          <t>YGR243W</t>
         </is>
       </c>
     </row>
@@ -3331,7 +3331,7 @@
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>YDR232W</t>
+          <t>YOL042W</t>
         </is>
       </c>
     </row>
@@ -3341,7 +3341,7 @@
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>YIL154C</t>
+          <t>YDR233C</t>
         </is>
       </c>
     </row>
@@ -3351,7 +3351,7 @@
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>YCL057C-A</t>
+          <t>YOR130C</t>
         </is>
       </c>
     </row>
@@ -3361,7 +3361,7 @@
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>YMR064W</t>
+          <t>YDR529C</t>
         </is>
       </c>
     </row>
@@ -3371,7 +3371,7 @@
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>YHL014C</t>
+          <t>YDL198C</t>
         </is>
       </c>
     </row>
@@ -3381,7 +3381,7 @@
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>YLR091W</t>
+          <t>YPL132W</t>
         </is>
       </c>
     </row>
@@ -3391,7 +3391,7 @@
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>YER014W</t>
+          <t>YKL134C</t>
         </is>
       </c>
     </row>
@@ -3401,7 +3401,7 @@
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>YJL023C</t>
+          <t>YOR100C</t>
         </is>
       </c>
     </row>
@@ -3411,7 +3411,7 @@
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>YDR350C</t>
+          <t>YLR283W</t>
         </is>
       </c>
     </row>
@@ -3421,7 +3421,7 @@
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>YMR108W</t>
+          <t>YPR058W</t>
         </is>
       </c>
     </row>
@@ -3431,7 +3431,7 @@
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>YNL098C</t>
+          <t>YMR098C</t>
         </is>
       </c>
     </row>
@@ -3441,7 +3441,7 @@
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>YKL003C</t>
+          <t>Q0120</t>
         </is>
       </c>
     </row>
@@ -3451,7 +3451,7 @@
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>YLR342W</t>
+          <t>YGL236C</t>
         </is>
       </c>
     </row>
@@ -3461,7 +3461,7 @@
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>YMR038C</t>
+          <t>YER014W</t>
         </is>
       </c>
     </row>
@@ -3471,7 +3471,7 @@
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>YDL174C</t>
+          <t>YER168C</t>
         </is>
       </c>
     </row>
@@ -3481,7 +3481,7 @@
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>YPR011C</t>
+          <t>YDR316W</t>
         </is>
       </c>
     </row>
@@ -3491,7 +3491,7 @@
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>YKR087C</t>
+          <t>YDR381C-A</t>
         </is>
       </c>
     </row>
@@ -3501,7 +3501,7 @@
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>YOR330C</t>
+          <t>YCL044C</t>
         </is>
       </c>
     </row>
@@ -3511,7 +3511,7 @@
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>YJR121W</t>
+          <t>YKL011C</t>
         </is>
       </c>
     </row>
@@ -3521,7 +3521,7 @@
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>YKL106W</t>
+          <t>Q0275</t>
         </is>
       </c>
     </row>
@@ -3531,7 +3531,7 @@
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>YMR307W</t>
+          <t>YPR021C</t>
         </is>
       </c>
     </row>
@@ -3541,7 +3541,7 @@
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>YDL217C</t>
+          <t>YER170W</t>
         </is>
       </c>
     </row>
@@ -3551,7 +3551,7 @@
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>YDR178W</t>
+          <t>YJL166W</t>
         </is>
       </c>
     </row>
@@ -3561,7 +3561,7 @@
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>YJL133W</t>
+          <t>YLR204W</t>
         </is>
       </c>
     </row>
@@ -3571,7 +3571,7 @@
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>YHR135C</t>
+          <t>YDR065W</t>
         </is>
       </c>
     </row>
@@ -3581,7 +3581,7 @@
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>YGR255C</t>
+          <t>YKL196C</t>
         </is>
       </c>
     </row>
@@ -3591,7 +3591,7 @@
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>YPL118W</t>
+          <t>YCR010C</t>
         </is>
       </c>
     </row>
@@ -3601,7 +3601,7 @@
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>YGR046W</t>
+          <t>YNL005C</t>
         </is>
       </c>
     </row>
@@ -3611,7 +3611,7 @@
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>YGL064C</t>
+          <t>YER125W</t>
         </is>
       </c>
     </row>
@@ -3621,7 +3621,7 @@
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>YDR237W</t>
+          <t>Q0065</t>
         </is>
       </c>
     </row>
@@ -3631,7 +3631,7 @@
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>YEL030W</t>
+          <t>YPL231W</t>
         </is>
       </c>
     </row>
@@ -3641,7 +3641,7 @@
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>YDL044C</t>
+          <t>YLR348C</t>
         </is>
       </c>
     </row>
@@ -3651,7 +3651,7 @@
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>YNR017W</t>
+          <t>YML081C-A</t>
         </is>
       </c>
     </row>
@@ -3661,7 +3661,7 @@
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>YBR251W</t>
+          <t>YPR134W</t>
         </is>
       </c>
     </row>
@@ -3671,7 +3671,7 @@
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>Q0160</t>
+          <t>YHR135C</t>
         </is>
       </c>
     </row>
@@ -3681,7 +3681,7 @@
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>YHL038C</t>
+          <t>YLR393W</t>
         </is>
       </c>
     </row>
@@ -3691,7 +3691,7 @@
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>YMR158W</t>
+          <t>YMR145C</t>
         </is>
       </c>
     </row>
@@ -3701,7 +3701,7 @@
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>YMR115W</t>
+          <t>Q0160</t>
         </is>
       </c>
     </row>
@@ -3711,7 +3711,7 @@
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>YAL039C</t>
+          <t>YFL036W</t>
         </is>
       </c>
     </row>
@@ -3721,7 +3721,7 @@
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>YGL107C</t>
+          <t>YDR061W</t>
         </is>
       </c>
     </row>
@@ -3731,7 +3731,7 @@
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>YGR033C</t>
+          <t>YBL030C</t>
         </is>
       </c>
     </row>
@@ -3741,7 +3741,7 @@
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t>YPR024W</t>
+          <t>YDR231C</t>
         </is>
       </c>
     </row>
@@ -3751,7 +3751,7 @@
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>YER077C</t>
+          <t>YML030W</t>
         </is>
       </c>
     </row>
@@ -3761,7 +3761,7 @@
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>YHR194W</t>
+          <t>YDR058C</t>
         </is>
       </c>
     </row>
@@ -3771,7 +3771,7 @@
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>YIL006W</t>
+          <t>YHL038C</t>
         </is>
       </c>
     </row>
@@ -3781,7 +3781,7 @@
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t>YOR305W</t>
+          <t>YGR220C</t>
         </is>
       </c>
     </row>
@@ -3791,7 +3791,7 @@
       </c>
       <c r="B337" t="inlineStr">
         <is>
-          <t>Q0065</t>
+          <t>YML025C</t>
         </is>
       </c>
     </row>
@@ -3801,7 +3801,7 @@
       </c>
       <c r="B338" t="inlineStr">
         <is>
-          <t>YML052W</t>
+          <t>YKL016C</t>
         </is>
       </c>
     </row>
@@ -3811,7 +3811,7 @@
       </c>
       <c r="B339" t="inlineStr">
         <is>
-          <t>YGR101W</t>
+          <t>YPR011C</t>
         </is>
       </c>
     </row>
@@ -3821,7 +3821,7 @@
       </c>
       <c r="B340" t="inlineStr">
         <is>
-          <t>YKL217W</t>
+          <t>YPR033C</t>
         </is>
       </c>
     </row>
@@ -3831,7 +3831,7 @@
       </c>
       <c r="B341" t="inlineStr">
         <is>
-          <t>YMR188C</t>
+          <t>YOR350C</t>
         </is>
       </c>
     </row>
@@ -3841,7 +3841,7 @@
       </c>
       <c r="B342" t="inlineStr">
         <is>
-          <t>YBR104W</t>
+          <t>YLR091W</t>
         </is>
       </c>
     </row>
@@ -3851,7 +3851,7 @@
       </c>
       <c r="B343" t="inlineStr">
         <is>
-          <t>YPL231W</t>
+          <t>YHR100C</t>
         </is>
       </c>
     </row>
@@ -3861,7 +3861,7 @@
       </c>
       <c r="B344" t="inlineStr">
         <is>
-          <t>YLR393W</t>
+          <t>YDR041W</t>
         </is>
       </c>
     </row>
@@ -3871,7 +3871,7 @@
       </c>
       <c r="B345" t="inlineStr">
         <is>
-          <t>YBR192W</t>
+          <t>YDR376W</t>
         </is>
       </c>
     </row>
@@ -3881,7 +3881,7 @@
       </c>
       <c r="B346" t="inlineStr">
         <is>
-          <t>YIL087C</t>
+          <t>Q0055</t>
         </is>
       </c>
     </row>
@@ -3891,7 +3891,7 @@
       </c>
       <c r="B347" t="inlineStr">
         <is>
-          <t>YBR039W</t>
+          <t>YNR045W</t>
         </is>
       </c>
     </row>
@@ -3901,7 +3901,7 @@
       </c>
       <c r="B348" t="inlineStr">
         <is>
-          <t>YBL099W</t>
+          <t>YER141W</t>
         </is>
       </c>
     </row>
@@ -3911,7 +3911,7 @@
       </c>
       <c r="B349" t="inlineStr">
         <is>
-          <t>YPL224C</t>
+          <t>YGR257C</t>
         </is>
       </c>
     </row>
@@ -3921,7 +3921,7 @@
       </c>
       <c r="B350" t="inlineStr">
         <is>
-          <t>YOR017W</t>
+          <t>YOR232W</t>
         </is>
       </c>
     </row>
@@ -3931,7 +3931,7 @@
       </c>
       <c r="B351" t="inlineStr">
         <is>
-          <t>YPL098C</t>
+          <t>YPR166C</t>
         </is>
       </c>
     </row>
@@ -3941,7 +3941,7 @@
       </c>
       <c r="B352" t="inlineStr">
         <is>
-          <t>YKL134C</t>
+          <t>YML110C</t>
         </is>
       </c>
     </row>
@@ -3951,7 +3951,7 @@
       </c>
       <c r="B353" t="inlineStr">
         <is>
-          <t>YML030W</t>
+          <t>YOR147W</t>
         </is>
       </c>
     </row>
@@ -3961,7 +3961,7 @@
       </c>
       <c r="B354" t="inlineStr">
         <is>
-          <t>YCL004W</t>
+          <t>YML052W</t>
         </is>
       </c>
     </row>
@@ -3971,7 +3971,7 @@
       </c>
       <c r="B355" t="inlineStr">
         <is>
-          <t>YOR020W-A</t>
+          <t>YER017C</t>
         </is>
       </c>
     </row>
@@ -3981,7 +3981,7 @@
       </c>
       <c r="B356" t="inlineStr">
         <is>
-          <t>YLR289W</t>
+          <t>YBR121C</t>
         </is>
       </c>
     </row>
@@ -3991,7 +3991,7 @@
       </c>
       <c r="B357" t="inlineStr">
         <is>
-          <t>YKL029C</t>
+          <t>YNL003C</t>
         </is>
       </c>
     </row>
@@ -4001,7 +4001,7 @@
       </c>
       <c r="B358" t="inlineStr">
         <is>
-          <t>YNL071W</t>
+          <t>YGL080W</t>
         </is>
       </c>
     </row>
@@ -4011,7 +4011,7 @@
       </c>
       <c r="B359" t="inlineStr">
         <is>
-          <t>YGR243W</t>
+          <t>YBR262C</t>
         </is>
       </c>
     </row>
@@ -4021,7 +4021,7 @@
       </c>
       <c r="B360" t="inlineStr">
         <is>
-          <t>YKL113C</t>
+          <t>YLR439W</t>
         </is>
       </c>
     </row>
@@ -4031,7 +4031,7 @@
       </c>
       <c r="B361" t="inlineStr">
         <is>
-          <t>YNL125C</t>
+          <t>YPL270W</t>
         </is>
       </c>
     </row>
@@ -4041,7 +4041,7 @@
       </c>
       <c r="B362" t="inlineStr">
         <is>
-          <t>YDR494W</t>
+          <t>YDR405W</t>
         </is>
       </c>
     </row>
@@ -4051,7 +4051,7 @@
       </c>
       <c r="B363" t="inlineStr">
         <is>
-          <t>YIL022W</t>
+          <t>YJL045W</t>
         </is>
       </c>
     </row>
@@ -4061,7 +4061,7 @@
       </c>
       <c r="B364" t="inlineStr">
         <is>
-          <t>YLR251W</t>
+          <t>YOR065W</t>
         </is>
       </c>
     </row>
@@ -4071,7 +4071,7 @@
       </c>
       <c r="B365" t="inlineStr">
         <is>
-          <t>YOL027C</t>
+          <t>YGR231C</t>
         </is>
       </c>
     </row>
@@ -4081,7 +4081,7 @@
       </c>
       <c r="B366" t="inlineStr">
         <is>
-          <t>YOR130C</t>
+          <t>YPL271W</t>
         </is>
       </c>
     </row>
@@ -4091,7 +4091,7 @@
       </c>
       <c r="B367" t="inlineStr">
         <is>
-          <t>YKL141W</t>
+          <t>YDR178W</t>
         </is>
       </c>
     </row>
@@ -4101,7 +4101,7 @@
       </c>
       <c r="B368" t="inlineStr">
         <is>
-          <t>YBR091C</t>
+          <t>YOR205C</t>
         </is>
       </c>
     </row>
@@ -4111,7 +4111,7 @@
       </c>
       <c r="B369" t="inlineStr">
         <is>
-          <t>YPR116W</t>
+          <t>YOR020W-A</t>
         </is>
       </c>
     </row>
@@ -4121,7 +4121,7 @@
       </c>
       <c r="B370" t="inlineStr">
         <is>
-          <t>YDL119C</t>
+          <t>YDL183C</t>
         </is>
       </c>
     </row>
@@ -4131,7 +4131,7 @@
       </c>
       <c r="B371" t="inlineStr">
         <is>
-          <t>YLR038C</t>
+          <t>YML091C</t>
         </is>
       </c>
     </row>
@@ -4141,7 +4141,7 @@
       </c>
       <c r="B372" t="inlineStr">
         <is>
-          <t>YML120C</t>
+          <t>YJR101W</t>
         </is>
       </c>
     </row>
@@ -4151,7 +4151,7 @@
       </c>
       <c r="B373" t="inlineStr">
         <is>
-          <t>YPL271W</t>
+          <t>YPL109C</t>
         </is>
       </c>
     </row>
@@ -4161,7 +4161,7 @@
       </c>
       <c r="B374" t="inlineStr">
         <is>
-          <t>YLR295C</t>
+          <t>YBR085W</t>
         </is>
       </c>
     </row>
@@ -4171,7 +4171,7 @@
       </c>
       <c r="B375" t="inlineStr">
         <is>
-          <t>Q0060</t>
+          <t>YNR041C</t>
         </is>
       </c>
     </row>
@@ -4181,7 +4181,7 @@
       </c>
       <c r="B376" t="inlineStr">
         <is>
-          <t>YBR044C</t>
+          <t>YGL119W</t>
         </is>
       </c>
     </row>
@@ -4191,7 +4191,7 @@
       </c>
       <c r="B377" t="inlineStr">
         <is>
-          <t>YCR046C</t>
+          <t>YDL044C</t>
         </is>
       </c>
     </row>
@@ -4201,7 +4201,7 @@
       </c>
       <c r="B378" t="inlineStr">
         <is>
-          <t>YNR018W</t>
+          <t>YER154W</t>
         </is>
       </c>
     </row>
@@ -4211,7 +4211,7 @@
       </c>
       <c r="B379" t="inlineStr">
         <is>
-          <t>YDR236C</t>
+          <t>Q0080</t>
         </is>
       </c>
     </row>
@@ -4221,7 +4221,7 @@
       </c>
       <c r="B380" t="inlineStr">
         <is>
-          <t>YFL036W</t>
+          <t>YMR097C</t>
         </is>
       </c>
     </row>
@@ -4231,7 +4231,7 @@
       </c>
       <c r="B381" t="inlineStr">
         <is>
-          <t>YLR193C</t>
+          <t>YDR197W</t>
         </is>
       </c>
     </row>
@@ -4241,7 +4241,7 @@
       </c>
       <c r="B382" t="inlineStr">
         <is>
-          <t>YLR253W</t>
+          <t>YMR307W</t>
         </is>
       </c>
     </row>
@@ -4251,7 +4251,7 @@
       </c>
       <c r="B383" t="inlineStr">
         <is>
-          <t>YDR079W</t>
+          <t>YJL133W</t>
         </is>
       </c>
     </row>
@@ -4261,7 +4261,7 @@
       </c>
       <c r="B384" t="inlineStr">
         <is>
-          <t>YDR033W</t>
+          <t>YIL006W</t>
         </is>
       </c>
     </row>
@@ -4271,7 +4271,7 @@
       </c>
       <c r="B385" t="inlineStr">
         <is>
-          <t>YJR077C</t>
+          <t>YLR067C</t>
         </is>
       </c>
     </row>
@@ -4281,7 +4281,7 @@
       </c>
       <c r="B386" t="inlineStr">
         <is>
-          <t>YLR390W</t>
+          <t>YDL085W</t>
         </is>
       </c>
     </row>
@@ -4291,7 +4291,7 @@
       </c>
       <c r="B387" t="inlineStr">
         <is>
-          <t>YPR058W</t>
+          <t>YHR199C</t>
         </is>
       </c>
     </row>
@@ -4301,7 +4301,7 @@
       </c>
       <c r="B388" t="inlineStr">
         <is>
-          <t>YNL306W</t>
+          <t>YCL009C</t>
         </is>
       </c>
     </row>
@@ -4311,7 +4311,7 @@
       </c>
       <c r="B389" t="inlineStr">
         <is>
-          <t>YPR134W</t>
+          <t>YDL119C</t>
         </is>
       </c>
     </row>
@@ -4321,7 +4321,7 @@
       </c>
       <c r="B390" t="inlineStr">
         <is>
-          <t>YLR077W</t>
+          <t>YGR101W</t>
         </is>
       </c>
     </row>
@@ -4331,7 +4331,7 @@
       </c>
       <c r="B391" t="inlineStr">
         <is>
-          <t>YCL017C</t>
+          <t>YLR295C</t>
         </is>
       </c>
     </row>
@@ -4341,7 +4341,7 @@
       </c>
       <c r="B392" t="inlineStr">
         <is>
-          <t>YKL195W</t>
+          <t>YIL155C</t>
         </is>
       </c>
     </row>
@@ -4351,7 +4351,7 @@
       </c>
       <c r="B393" t="inlineStr">
         <is>
-          <t>YMR145C</t>
+          <t>YBR047W</t>
         </is>
       </c>
     </row>
@@ -4361,7 +4361,7 @@
       </c>
       <c r="B394" t="inlineStr">
         <is>
-          <t>YOR356W</t>
+          <t>YJL171C</t>
         </is>
       </c>
     </row>
@@ -4371,7 +4371,7 @@
       </c>
       <c r="B395" t="inlineStr">
         <is>
-          <t>YDR061W</t>
+          <t>YER080W</t>
         </is>
       </c>
     </row>
@@ -4381,7 +4381,7 @@
       </c>
       <c r="B396" t="inlineStr">
         <is>
-          <t>YOR196C</t>
+          <t>YGR183C</t>
         </is>
       </c>
     </row>
@@ -4391,7 +4391,7 @@
       </c>
       <c r="B397" t="inlineStr">
         <is>
-          <t>YOR125C</t>
+          <t>YKL170W</t>
         </is>
       </c>
     </row>
@@ -4401,7 +4401,7 @@
       </c>
       <c r="B398" t="inlineStr">
         <is>
-          <t>YDR322C-A</t>
+          <t>YKL120W</t>
         </is>
       </c>
     </row>
@@ -4411,7 +4411,7 @@
       </c>
       <c r="B399" t="inlineStr">
         <is>
-          <t>YKL196C</t>
+          <t>YOR356W</t>
         </is>
       </c>
     </row>
@@ -4421,7 +4421,7 @@
       </c>
       <c r="B400" t="inlineStr">
         <is>
-          <t>YGR222W</t>
+          <t>YKR065C</t>
         </is>
       </c>
     </row>
@@ -4431,7 +4431,7 @@
       </c>
       <c r="B401" t="inlineStr">
         <is>
-          <t>YGR165W</t>
+          <t>Q0060</t>
         </is>
       </c>
     </row>
@@ -4441,7 +4441,7 @@
       </c>
       <c r="B402" t="inlineStr">
         <is>
-          <t>YIR021W</t>
+          <t>YLR008C</t>
         </is>
       </c>
     </row>
@@ -4451,7 +4451,7 @@
       </c>
       <c r="B403" t="inlineStr">
         <is>
-          <t>YDR529C</t>
+          <t>YJL063C</t>
         </is>
       </c>
     </row>
@@ -4461,7 +4461,7 @@
       </c>
       <c r="B404" t="inlineStr">
         <is>
-          <t>YDL069C</t>
+          <t>YOR266W</t>
         </is>
       </c>
     </row>
@@ -4471,7 +4471,7 @@
       </c>
       <c r="B405" t="inlineStr">
         <is>
-          <t>YLR204W</t>
+          <t>YLR059C</t>
         </is>
       </c>
     </row>
@@ -4481,7 +4481,7 @@
       </c>
       <c r="B406" t="inlineStr">
         <is>
-          <t>YCL044C</t>
+          <t>YCR004C</t>
         </is>
       </c>
     </row>
@@ -4491,7 +4491,7 @@
       </c>
       <c r="B407" t="inlineStr">
         <is>
-          <t>YPL134C</t>
+          <t>YMR301C</t>
         </is>
       </c>
     </row>
@@ -4501,7 +4501,7 @@
       </c>
       <c r="B408" t="inlineStr">
         <is>
-          <t>YPL270W</t>
+          <t>YGL064C</t>
         </is>
       </c>
     </row>
@@ -4511,7 +4511,7 @@
       </c>
       <c r="B409" t="inlineStr">
         <is>
-          <t>YMR301C</t>
+          <t>YLR038C</t>
         </is>
       </c>
     </row>
@@ -4521,7 +4521,7 @@
       </c>
       <c r="B410" t="inlineStr">
         <is>
-          <t>YEL024W</t>
+          <t>YOR271C</t>
         </is>
       </c>
     </row>
@@ -4531,7 +4531,7 @@
       </c>
       <c r="B411" t="inlineStr">
         <is>
-          <t>YJL147C</t>
+          <t>YPL098C</t>
         </is>
       </c>
     </row>
@@ -4541,7 +4541,7 @@
       </c>
       <c r="B412" t="inlineStr">
         <is>
-          <t>YLR283W</t>
+          <t>YGR132C</t>
         </is>
       </c>
     </row>
@@ -4551,7 +4551,7 @@
       </c>
       <c r="B413" t="inlineStr">
         <is>
-          <t>YDR462W</t>
+          <t>YOR222W</t>
         </is>
       </c>
     </row>
@@ -4561,7 +4561,7 @@
       </c>
       <c r="B414" t="inlineStr">
         <is>
-          <t>YGR147C</t>
+          <t>YNL098C</t>
         </is>
       </c>
     </row>
@@ -4571,7 +4571,7 @@
       </c>
       <c r="B415" t="inlineStr">
         <is>
-          <t>YKR016W</t>
+          <t>YOL059W</t>
         </is>
       </c>
     </row>
@@ -4581,7 +4581,7 @@
       </c>
       <c r="B416" t="inlineStr">
         <is>
-          <t>YDL198C</t>
+          <t>YKR087C</t>
         </is>
       </c>
     </row>
@@ -4591,7 +4591,7 @@
       </c>
       <c r="B417" t="inlineStr">
         <is>
-          <t>YGR132C</t>
+          <t>YHR001W-A</t>
         </is>
       </c>
     </row>
@@ -4601,7 +4601,7 @@
       </c>
       <c r="B418" t="inlineStr">
         <is>
-          <t>YER141W</t>
+          <t>YDL217C</t>
         </is>
       </c>
     </row>
@@ -4611,7 +4611,7 @@
       </c>
       <c r="B419" t="inlineStr">
         <is>
-          <t>YKL133C</t>
+          <t>YKL113C</t>
         </is>
       </c>
     </row>
@@ -4621,7 +4621,7 @@
       </c>
       <c r="B420" t="inlineStr">
         <is>
-          <t>YDR377W</t>
+          <t>YKL187C</t>
         </is>
       </c>
     </row>
@@ -4631,7 +4631,7 @@
       </c>
       <c r="B421" t="inlineStr">
         <is>
-          <t>YPL132W</t>
+          <t>YBR054W</t>
         </is>
       </c>
     </row>
@@ -4641,7 +4641,7 @@
       </c>
       <c r="B422" t="inlineStr">
         <is>
-          <t>YER153C</t>
+          <t>YDR236C</t>
         </is>
       </c>
     </row>
@@ -4651,7 +4651,7 @@
       </c>
       <c r="B423" t="inlineStr">
         <is>
-          <t>YMR228W</t>
+          <t>YML129C</t>
         </is>
       </c>
     </row>
@@ -4661,7 +4661,7 @@
       </c>
       <c r="B424" t="inlineStr">
         <is>
-          <t>YPR191W</t>
+          <t>YKL141W</t>
         </is>
       </c>
     </row>
@@ -4671,7 +4671,7 @@
       </c>
       <c r="B425" t="inlineStr">
         <is>
-          <t>YIL105C</t>
+          <t>YBL022C</t>
         </is>
       </c>
     </row>
@@ -4681,7 +4681,7 @@
       </c>
       <c r="B426" t="inlineStr">
         <is>
-          <t>YPR140W</t>
+          <t>YKL056C</t>
         </is>
       </c>
     </row>
@@ -4691,7 +4691,7 @@
       </c>
       <c r="B427" t="inlineStr">
         <is>
-          <t>YGL129C</t>
+          <t>YIL134W</t>
         </is>
       </c>
     </row>
@@ -4701,7 +4701,7 @@
       </c>
       <c r="B428" t="inlineStr">
         <is>
-          <t>YDR194C</t>
+          <t>YPR140W</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: add new files
</commit_message>
<xml_diff>
--- a/data/sce_compartment_curation/mitochondrial_inner_membrane_annotations_manual_v3.xlsx
+++ b/data/sce_compartment_curation/mitochondrial_inner_membrane_annotations_manual_v3.xlsx
@@ -441,7 +441,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>YGR255C</t>
+          <t>YFR033C</t>
         </is>
       </c>
     </row>
@@ -451,7 +451,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>YDR185C</t>
+          <t>YLR382C</t>
         </is>
       </c>
     </row>
@@ -461,7 +461,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Q0160</t>
+          <t>YDL207W</t>
         </is>
       </c>
     </row>
@@ -471,7 +471,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>YER141W</t>
+          <t>YGL107C</t>
         </is>
       </c>
     </row>
@@ -481,7 +481,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Q0080</t>
+          <t>YOR086C</t>
         </is>
       </c>
     </row>
@@ -491,7 +491,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Q0275</t>
+          <t>YOR266W</t>
         </is>
       </c>
     </row>
@@ -501,7 +501,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>YBR039W</t>
+          <t>YKL087C</t>
         </is>
       </c>
     </row>
@@ -511,7 +511,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>YMR193W</t>
+          <t>YPL172C</t>
         </is>
       </c>
     </row>
@@ -521,7 +521,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>YGR112W</t>
+          <t>YBR078W</t>
         </is>
       </c>
     </row>
@@ -531,7 +531,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>YNL122C</t>
+          <t>YJR034W</t>
         </is>
       </c>
     </row>
@@ -541,7 +541,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>YDL142C</t>
+          <t>YDR375C</t>
         </is>
       </c>
     </row>
@@ -551,7 +551,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>YNL100W</t>
+          <t>YBR044C</t>
         </is>
       </c>
     </row>
@@ -561,7 +561,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>YMR228W</t>
+          <t>YDL004W</t>
         </is>
       </c>
     </row>
@@ -571,7 +571,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>YBR227C</t>
+          <t>YBL099W</t>
         </is>
       </c>
     </row>
@@ -581,7 +581,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>YMR212C</t>
+          <t>YHL038C</t>
         </is>
       </c>
     </row>
@@ -591,7 +591,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>YPR033C</t>
+          <t>YIL134W</t>
         </is>
       </c>
     </row>
@@ -601,7 +601,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>YNL185C</t>
+          <t>YLR283W</t>
         </is>
       </c>
     </row>
@@ -611,7 +611,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>YNL169C</t>
+          <t>YDR116C</t>
         </is>
       </c>
     </row>
@@ -621,7 +621,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>YDR393W</t>
+          <t>YDR298C</t>
         </is>
       </c>
     </row>
@@ -631,7 +631,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>YEL030W</t>
+          <t>YOL059W</t>
         </is>
       </c>
     </row>
@@ -641,7 +641,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>YLR239C</t>
+          <t>YOL042W</t>
         </is>
       </c>
     </row>
@@ -651,7 +651,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>YPL134C</t>
+          <t>YDR033W</t>
         </is>
       </c>
     </row>
@@ -661,7 +661,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>YIL105C</t>
+          <t>YPL231W</t>
         </is>
       </c>
     </row>
@@ -671,7 +671,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>YGL136C</t>
+          <t>YML030W</t>
         </is>
       </c>
     </row>
@@ -681,7 +681,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>YGR046W</t>
+          <t>YHR199C</t>
         </is>
       </c>
     </row>
@@ -691,7 +691,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>YBR163W</t>
+          <t>YGR231C</t>
         </is>
       </c>
     </row>
@@ -701,7 +701,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>YKL195W</t>
+          <t>YGL191W</t>
         </is>
       </c>
     </row>
@@ -711,7 +711,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>YDR384C</t>
+          <t>YOR232W</t>
         </is>
       </c>
     </row>
@@ -721,7 +721,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>YDL004W</t>
+          <t>YDR041W</t>
         </is>
       </c>
     </row>
@@ -731,7 +731,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>YPR191W</t>
+          <t>YLR204W</t>
         </is>
       </c>
     </row>
@@ -741,7 +741,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>YOR065W</t>
+          <t>YGL057C</t>
         </is>
       </c>
     </row>
@@ -751,7 +751,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>YER014W</t>
+          <t>YER166W</t>
         </is>
       </c>
     </row>
@@ -761,7 +761,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>YKR042W</t>
+          <t>YGR222W</t>
         </is>
       </c>
     </row>
@@ -771,7 +771,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>YOL053W</t>
+          <t>YCR046C</t>
         </is>
       </c>
     </row>
@@ -781,7 +781,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>YDL198C</t>
+          <t>YER182W</t>
         </is>
       </c>
     </row>
@@ -791,7 +791,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>YKL208W</t>
+          <t>YOL027C</t>
         </is>
       </c>
     </row>
@@ -801,7 +801,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>YML025C</t>
+          <t>YML128C</t>
         </is>
       </c>
     </row>
@@ -811,7 +811,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>YDR032C</t>
+          <t>YCL009C</t>
         </is>
       </c>
     </row>
@@ -821,7 +821,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>YGR116W</t>
+          <t>YJR101W</t>
         </is>
       </c>
     </row>
@@ -831,7 +831,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>YML128C</t>
+          <t>YPR125W</t>
         </is>
       </c>
     </row>
@@ -841,7 +841,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>YDL044C</t>
+          <t>YNR002C</t>
         </is>
       </c>
     </row>
@@ -851,7 +851,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>YNL003C</t>
+          <t>YLR239C</t>
         </is>
       </c>
     </row>
@@ -861,7 +861,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>YLR253W</t>
+          <t>YPR191W</t>
         </is>
       </c>
     </row>
@@ -871,7 +871,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>YER170W</t>
+          <t>YKL138C</t>
         </is>
       </c>
     </row>
@@ -881,7 +881,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>YKL087C</t>
+          <t>YBR037C</t>
         </is>
       </c>
     </row>
@@ -891,7 +891,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>YCR046C</t>
+          <t>YGL080W</t>
         </is>
       </c>
     </row>
@@ -901,7 +901,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>YMR064W</t>
+          <t>YGR112W</t>
         </is>
       </c>
     </row>
@@ -911,7 +911,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>YMR056C</t>
+          <t>YHR135C</t>
         </is>
       </c>
     </row>
@@ -921,7 +921,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>YOR201C</t>
+          <t>YAL054C</t>
         </is>
       </c>
     </row>
@@ -931,7 +931,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>YHR198C</t>
+          <t>YIL006W</t>
         </is>
       </c>
     </row>
@@ -941,7 +941,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>YPR011C</t>
+          <t>YMR038C</t>
         </is>
       </c>
     </row>
@@ -951,7 +951,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>YPL098C</t>
+          <t>YGL119W</t>
         </is>
       </c>
     </row>
@@ -961,7 +961,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>YHR001W-A</t>
+          <t>YPL063W</t>
         </is>
       </c>
     </row>
@@ -971,7 +971,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>YFL036W</t>
+          <t>YHL014C</t>
         </is>
       </c>
     </row>
@@ -981,7 +981,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>YDL215C</t>
+          <t>YLR193C</t>
         </is>
       </c>
     </row>
@@ -991,7 +991,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>YIL022W</t>
+          <t>YMR177W</t>
         </is>
       </c>
     </row>
@@ -1001,7 +1001,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>YBL099W</t>
+          <t>YDR233C</t>
         </is>
       </c>
     </row>
@@ -1011,7 +1011,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>YBR291C</t>
+          <t>YJL102W</t>
         </is>
       </c>
     </row>
@@ -1031,7 +1031,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>YBR024W</t>
+          <t>YPR061C</t>
         </is>
       </c>
     </row>
@@ -1041,7 +1041,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>YGR193C</t>
+          <t>YOL095C</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>YKL029C</t>
+          <t>YMR302C</t>
         </is>
       </c>
     </row>
@@ -1061,7 +1061,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>YKL170W</t>
+          <t>YLL041C</t>
         </is>
       </c>
     </row>
@@ -1071,7 +1071,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Q0105</t>
+          <t>YIL077C</t>
         </is>
       </c>
     </row>
@@ -1081,7 +1081,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>YPL118W</t>
+          <t>YJR121W</t>
         </is>
       </c>
     </row>
@@ -1091,7 +1091,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>YOR354C</t>
+          <t>YKR065C</t>
         </is>
       </c>
     </row>
@@ -1101,7 +1101,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>YOR147W</t>
+          <t>YNR045W</t>
         </is>
       </c>
     </row>
@@ -1111,7 +1111,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Q0065</t>
+          <t>YNL100W</t>
         </is>
       </c>
     </row>
@@ -1121,7 +1121,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>YKR016W</t>
+          <t>YGR165W</t>
         </is>
       </c>
     </row>
@@ -1131,7 +1131,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>YML072C</t>
+          <t>YGR236C</t>
         </is>
       </c>
     </row>
@@ -1141,7 +1141,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>YGR171C</t>
+          <t>Q0105</t>
         </is>
       </c>
     </row>
@@ -1151,7 +1151,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>YGR150C</t>
+          <t>YNL122C</t>
         </is>
       </c>
     </row>
@@ -1161,7 +1161,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>YJL054W</t>
+          <t>YBR282W</t>
         </is>
       </c>
     </row>
@@ -1171,7 +1171,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>YKR052C</t>
+          <t>YLR312W-A</t>
         </is>
       </c>
     </row>
@@ -1181,7 +1181,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>YIL154C</t>
+          <t>YJL209W</t>
         </is>
       </c>
     </row>
@@ -1191,7 +1191,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>YLR193C</t>
+          <t>YNL211C</t>
         </is>
       </c>
     </row>
@@ -1201,7 +1201,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>YMR145C</t>
+          <t>YOR065W</t>
         </is>
       </c>
     </row>
@@ -1211,7 +1211,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Q0120</t>
+          <t>YJL143W</t>
         </is>
       </c>
     </row>
@@ -1221,7 +1221,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>YHR005C-A</t>
+          <t>YPL168W</t>
         </is>
       </c>
     </row>
@@ -1231,7 +1231,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>YHR002W</t>
+          <t>YGR220C</t>
         </is>
       </c>
     </row>
@@ -1241,7 +1241,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>YJR121W</t>
+          <t>YLR139C</t>
         </is>
       </c>
     </row>
@@ -1251,7 +1251,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>YGR132C</t>
+          <t>YKL141W</t>
         </is>
       </c>
     </row>
@@ -1261,7 +1261,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>YJL045W</t>
+          <t>YKR042W</t>
         </is>
       </c>
     </row>
@@ -1271,7 +1271,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>YBR044C</t>
+          <t>YDR494W</t>
         </is>
       </c>
     </row>
@@ -1281,7 +1281,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Q0050</t>
+          <t>YJL133W</t>
         </is>
       </c>
     </row>
@@ -1291,7 +1291,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>YDR237W</t>
+          <t>YKL055C</t>
         </is>
       </c>
     </row>
@@ -1301,7 +1301,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>YNL177C</t>
+          <t>YOR130C</t>
         </is>
       </c>
     </row>
@@ -1311,7 +1311,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>YGR147C</t>
+          <t>YDR376W</t>
         </is>
       </c>
     </row>
@@ -1321,7 +1321,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>YGR222W</t>
+          <t>Q0045</t>
         </is>
       </c>
     </row>
@@ -1331,7 +1331,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>YJR034W</t>
+          <t>YER058W</t>
         </is>
       </c>
     </row>
@@ -1341,7 +1341,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>YML110C</t>
+          <t>YOR100C</t>
         </is>
       </c>
     </row>
@@ -1351,7 +1351,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>YPL270W</t>
+          <t>Q0110</t>
         </is>
       </c>
     </row>
@@ -1361,7 +1361,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>YDR322C-A</t>
+          <t>YDR032C</t>
         </is>
       </c>
     </row>
@@ -1371,7 +1371,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>YPR061C</t>
+          <t>YIL111W</t>
         </is>
       </c>
     </row>
@@ -1381,7 +1381,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>YGR243W</t>
+          <t>YIL016W</t>
         </is>
       </c>
     </row>
@@ -1391,7 +1391,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>YNL052W</t>
+          <t>YFL046W</t>
         </is>
       </c>
     </row>
@@ -1401,7 +1401,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>YBR078W</t>
+          <t>YKL113C</t>
         </is>
       </c>
     </row>
@@ -1411,7 +1411,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>YPL103C</t>
+          <t>YER154W</t>
         </is>
       </c>
     </row>
@@ -1421,7 +1421,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>YBR104W</t>
+          <t>YDR058C</t>
         </is>
       </c>
     </row>
@@ -1431,7 +1431,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>YBL013W</t>
+          <t>YML091C</t>
         </is>
       </c>
     </row>
@@ -1441,7 +1441,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>YDR282C</t>
+          <t>YLR091W</t>
         </is>
       </c>
     </row>
@@ -1451,7 +1451,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>YLR312W-A</t>
+          <t>YHR002W</t>
         </is>
       </c>
     </row>
@@ -1461,7 +1461,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>YDL183C</t>
+          <t>YHR198C</t>
         </is>
       </c>
     </row>
@@ -1471,7 +1471,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>YHR011W</t>
+          <t>YPL132W</t>
         </is>
       </c>
     </row>
@@ -1481,7 +1481,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>YMR098C</t>
+          <t>YBL022C</t>
         </is>
       </c>
     </row>
@@ -1491,7 +1491,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>YLR390W</t>
+          <t>YPL271W</t>
         </is>
       </c>
     </row>
@@ -1501,7 +1501,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>YOR221C</t>
+          <t>YGL226W</t>
         </is>
       </c>
     </row>
@@ -1511,7 +1511,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>YDR058C</t>
+          <t>YOR176W</t>
         </is>
       </c>
     </row>
@@ -1521,7 +1521,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>YNL098C</t>
+          <t>YDR232W</t>
         </is>
       </c>
     </row>
@@ -1531,7 +1531,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>YPR024W</t>
+          <t>YNR041C</t>
         </is>
       </c>
     </row>
@@ -1541,7 +1541,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>YFR033C</t>
+          <t>YKR087C</t>
         </is>
       </c>
     </row>
@@ -1551,7 +1551,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>YML052W</t>
+          <t>YDR178W</t>
         </is>
       </c>
     </row>
@@ -1561,7 +1561,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>YDR197W</t>
+          <t>YNL177C</t>
         </is>
       </c>
     </row>
@@ -1571,7 +1571,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>YDL164C</t>
+          <t>YKL170W</t>
         </is>
       </c>
     </row>
@@ -1581,7 +1581,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>YOR086C</t>
+          <t>YBR024W</t>
         </is>
       </c>
     </row>
@@ -1591,7 +1591,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>YOL027C</t>
+          <t>YGL136C</t>
         </is>
       </c>
     </row>
@@ -1601,7 +1601,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>YOR196C</t>
+          <t>YBL095W</t>
         </is>
       </c>
     </row>
@@ -1611,7 +1611,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>YDL217C</t>
+          <t>YNL256W</t>
         </is>
       </c>
     </row>
@@ -1621,7 +1621,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>YOR037W</t>
+          <t>YLR295C</t>
         </is>
       </c>
     </row>
@@ -1631,7 +1631,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>YOL095C</t>
+          <t>YIL155C</t>
         </is>
       </c>
     </row>
@@ -1641,7 +1641,7 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>YDR079W</t>
+          <t>YNL169C</t>
         </is>
       </c>
     </row>
@@ -1651,7 +1651,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>YNL137C</t>
+          <t>YGR255C</t>
         </is>
       </c>
     </row>
@@ -1661,7 +1661,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>YMR066W</t>
+          <t>YDR231C</t>
         </is>
       </c>
     </row>
@@ -1671,7 +1671,7 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>YDL085W</t>
+          <t>YIL042C</t>
         </is>
       </c>
     </row>
@@ -1681,7 +1681,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>YOR330C</t>
+          <t>YOR037W</t>
         </is>
       </c>
     </row>
@@ -1691,7 +1691,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>YDL069C</t>
+          <t>YPR011C</t>
         </is>
       </c>
     </row>
@@ -1701,7 +1701,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>YGL107C</t>
+          <t>YNL009W</t>
         </is>
       </c>
     </row>
@@ -1711,7 +1711,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>YIL157C</t>
+          <t>YLR067C</t>
         </is>
       </c>
     </row>
@@ -1721,7 +1721,7 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>YLR348C</t>
+          <t>YHR194W</t>
         </is>
       </c>
     </row>
@@ -1731,7 +1731,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>YGR236C</t>
+          <t>YHR011W</t>
         </is>
       </c>
     </row>
@@ -1741,7 +1741,7 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>YJR101W</t>
+          <t>YER069W</t>
         </is>
       </c>
     </row>
@@ -1751,7 +1751,7 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>YCL057C-A</t>
+          <t>YDR065W</t>
         </is>
       </c>
     </row>
@@ -1761,7 +1761,7 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>YLR382C</t>
+          <t>YKL133C</t>
         </is>
       </c>
     </row>
@@ -1771,7 +1771,7 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>YIL087C</t>
+          <t>YJL208C</t>
         </is>
       </c>
     </row>
@@ -1781,7 +1781,7 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>YDL207W</t>
+          <t>YKL056C</t>
         </is>
       </c>
     </row>
@@ -1791,7 +1791,7 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>YOR017W</t>
+          <t>Q0160</t>
         </is>
       </c>
     </row>
@@ -1801,7 +1801,7 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>YDL027C</t>
+          <t>YKL148C</t>
         </is>
       </c>
     </row>
@@ -1811,7 +1811,7 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>YER019W</t>
+          <t>YIL157C</t>
         </is>
       </c>
     </row>
@@ -1821,7 +1821,7 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>YGL236C</t>
+          <t>YER141W</t>
         </is>
       </c>
     </row>
@@ -1831,7 +1831,7 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>Q0250</t>
+          <t>YGR101W</t>
         </is>
       </c>
     </row>
@@ -1841,7 +1841,7 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>YJR100C</t>
+          <t>YER170W</t>
         </is>
       </c>
     </row>
@@ -1851,7 +1851,7 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>YBR121C</t>
+          <t>YKR052C</t>
         </is>
       </c>
     </row>
@@ -1861,7 +1861,7 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>YAL054C</t>
+          <t>YDL174C</t>
         </is>
       </c>
     </row>
@@ -1871,7 +1871,7 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>YIL134W</t>
+          <t>YJR045C</t>
         </is>
       </c>
     </row>
@@ -1881,7 +1881,7 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>YPL271W</t>
+          <t>YLR188W</t>
         </is>
       </c>
     </row>
@@ -1891,7 +1891,7 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>YBR091C</t>
+          <t>YIL087C</t>
         </is>
       </c>
     </row>
@@ -1901,7 +1901,7 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>YHR199C</t>
+          <t>Q0060</t>
         </is>
       </c>
     </row>
@@ -1911,7 +1911,7 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>YOR205C</t>
+          <t>YER168C</t>
         </is>
       </c>
     </row>
@@ -1921,7 +1921,7 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>YFL016C</t>
+          <t>YPL078C</t>
         </is>
       </c>
     </row>
@@ -1931,7 +1931,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>YJR080C</t>
+          <t>YGR243W</t>
         </is>
       </c>
     </row>
@@ -1941,7 +1941,7 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>YHR147C</t>
+          <t>YNR018W</t>
         </is>
       </c>
     </row>
@@ -1951,7 +1951,7 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>YBR003W</t>
+          <t>YDL222C</t>
         </is>
       </c>
     </row>
@@ -1961,7 +1961,7 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>YPL132W</t>
+          <t>YGR116W</t>
         </is>
       </c>
     </row>
@@ -1971,7 +1971,7 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>YER069W</t>
+          <t>YOR211C</t>
         </is>
       </c>
     </row>
@@ -1981,7 +1981,7 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>YLR283W</t>
+          <t>YEL020W-A</t>
         </is>
       </c>
     </row>
@@ -1991,7 +1991,7 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>YMR150C</t>
+          <t>YER153C</t>
         </is>
       </c>
     </row>
@@ -2001,7 +2001,7 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>YNL328C</t>
+          <t>YGR183C</t>
         </is>
       </c>
     </row>
@@ -2011,7 +2011,7 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>YER154W</t>
+          <t>YHL004W</t>
         </is>
       </c>
     </row>
@@ -2021,7 +2021,7 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>YMR158W</t>
+          <t>YNL003C</t>
         </is>
       </c>
     </row>
@@ -2031,7 +2031,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>YKL148C</t>
+          <t>YLR090W</t>
         </is>
       </c>
     </row>
@@ -2041,7 +2041,7 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>YMR097C</t>
+          <t>YOR196C</t>
         </is>
       </c>
     </row>
@@ -2051,7 +2051,7 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>YGR220C</t>
+          <t>YDL217C</t>
         </is>
       </c>
     </row>
@@ -2061,7 +2061,7 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>YCR010C</t>
+          <t>YEL006W</t>
         </is>
       </c>
     </row>
@@ -2071,7 +2071,7 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>YCL004W</t>
+          <t>Q0065</t>
         </is>
       </c>
     </row>
@@ -2081,7 +2081,7 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>YBL095W</t>
+          <t>Q0080</t>
         </is>
       </c>
     </row>
@@ -2091,7 +2091,7 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>YDL174C</t>
+          <t>YOR354C</t>
         </is>
       </c>
     </row>
@@ -2101,7 +2101,7 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>YDR061W</t>
+          <t>YGL129C</t>
         </is>
       </c>
     </row>
@@ -2111,7 +2111,7 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>YNL005C</t>
+          <t>YLR393W</t>
         </is>
       </c>
     </row>
@@ -2121,7 +2121,7 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>YMR038C</t>
+          <t>YGR150C</t>
         </is>
       </c>
     </row>
@@ -2131,7 +2131,7 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>YNR018W</t>
+          <t>YLR342W</t>
         </is>
       </c>
     </row>
@@ -2141,7 +2141,7 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>YOR232W</t>
+          <t>YOR356W</t>
         </is>
       </c>
     </row>
@@ -2151,7 +2151,7 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>YEL020W-A</t>
+          <t>YMR257C</t>
         </is>
       </c>
     </row>
@@ -2161,7 +2161,7 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>YLR295C</t>
+          <t>YDR237W</t>
         </is>
       </c>
     </row>
@@ -2171,7 +2171,7 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>YLR188W</t>
+          <t>YMR089C</t>
         </is>
       </c>
     </row>
@@ -2181,7 +2181,7 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>Q0130</t>
+          <t>YGR062C</t>
         </is>
       </c>
     </row>
@@ -2191,7 +2191,7 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>YMR257C</t>
+          <t>Q0085</t>
         </is>
       </c>
     </row>
@@ -2201,7 +2201,7 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>YFL046W</t>
+          <t>YER014W</t>
         </is>
       </c>
     </row>
@@ -2211,7 +2211,7 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>YDR376W</t>
+          <t>YBR104W</t>
         </is>
       </c>
     </row>
@@ -2221,7 +2221,7 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>YER125W</t>
+          <t>YMR145C</t>
         </is>
       </c>
     </row>
@@ -2231,7 +2231,7 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>YLR290C</t>
+          <t>YPR140W</t>
         </is>
       </c>
     </row>
@@ -2241,7 +2241,7 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>YJL062W-A</t>
+          <t>YCL004W</t>
         </is>
       </c>
     </row>
@@ -2251,7 +2251,7 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>YBR084W</t>
+          <t>YMR256C</t>
         </is>
       </c>
     </row>
@@ -2261,7 +2261,7 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>Q0055</t>
+          <t>YGL059W</t>
         </is>
       </c>
     </row>
@@ -2271,7 +2271,7 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>YOL008W</t>
+          <t>YDR119W-A</t>
         </is>
       </c>
     </row>
@@ -2281,7 +2281,7 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>YOR125C</t>
+          <t>YOL023W</t>
         </is>
       </c>
     </row>
@@ -2291,7 +2291,7 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>YBL030C</t>
+          <t>YKL217W</t>
         </is>
       </c>
     </row>
@@ -2301,7 +2301,7 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>YLR395C</t>
+          <t>YLR008C</t>
         </is>
       </c>
     </row>
@@ -2311,7 +2311,7 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>YBR047W</t>
+          <t>YMR066W</t>
         </is>
       </c>
     </row>
@@ -2321,7 +2321,7 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>YNL009W</t>
+          <t>YNR040W</t>
         </is>
       </c>
     </row>
@@ -2331,7 +2331,7 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>YDL202W</t>
+          <t>YMR282C</t>
         </is>
       </c>
     </row>
@@ -2341,7 +2341,7 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>YCL044C</t>
+          <t>YER183C</t>
         </is>
       </c>
     </row>
@@ -2351,7 +2351,7 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>YER183C</t>
+          <t>YBR291C</t>
         </is>
       </c>
     </row>
@@ -2361,7 +2361,7 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>YJL147C</t>
+          <t>YKL155C</t>
         </is>
       </c>
     </row>
@@ -2371,7 +2371,7 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>YMR024W</t>
+          <t>YPR134W</t>
         </is>
       </c>
     </row>
@@ -2381,7 +2381,7 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>YLR077W</t>
+          <t>YDL119C</t>
         </is>
       </c>
     </row>
@@ -2391,7 +2391,7 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>YJL143W</t>
+          <t>YDL215C</t>
         </is>
       </c>
     </row>
@@ -2401,7 +2401,7 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>YGR096W</t>
+          <t>YML072C</t>
         </is>
       </c>
     </row>
@@ -2411,7 +2411,7 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>YLR084C</t>
+          <t>YOR205C</t>
         </is>
       </c>
     </row>
@@ -2421,7 +2421,7 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>YOR356W</t>
+          <t>Q0055</t>
         </is>
       </c>
     </row>
@@ -2431,7 +2431,7 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>YGR101W</t>
+          <t>YKL196C</t>
         </is>
       </c>
     </row>
@@ -2441,7 +2441,7 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>YGL119W</t>
+          <t>YMR228W</t>
         </is>
       </c>
     </row>
@@ -2451,7 +2451,7 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>YLR164W</t>
+          <t>YPR166C</t>
         </is>
       </c>
     </row>
@@ -2461,7 +2461,7 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>YPL029W</t>
+          <t>YDR393W</t>
         </is>
       </c>
     </row>
@@ -2471,7 +2471,7 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>YDR347W</t>
+          <t>YLR348C</t>
         </is>
       </c>
     </row>
@@ -2481,7 +2481,7 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>YKL141W</t>
+          <t>YMR150C</t>
         </is>
       </c>
     </row>
@@ -2491,7 +2491,7 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>YJL102W</t>
+          <t>YIR021W</t>
         </is>
       </c>
     </row>
@@ -2501,7 +2501,7 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>YDR405W</t>
+          <t>YFL036W</t>
         </is>
       </c>
     </row>
@@ -2511,7 +2511,7 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>YOR020W-A</t>
+          <t>YDR347W</t>
         </is>
       </c>
     </row>
@@ -2521,7 +2521,7 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>YOR100C</t>
+          <t>YBL045C</t>
         </is>
       </c>
     </row>
@@ -2531,7 +2531,7 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>YDR316W</t>
+          <t>YOR125C</t>
         </is>
       </c>
     </row>
@@ -2541,7 +2541,7 @@
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>YDR322W</t>
+          <t>YNL137C</t>
         </is>
       </c>
     </row>
@@ -2551,7 +2551,7 @@
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>YER182W</t>
+          <t>YDR350C</t>
         </is>
       </c>
     </row>
@@ -2561,7 +2561,7 @@
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>YPL060W</t>
+          <t>YPL098C</t>
         </is>
       </c>
     </row>
@@ -2571,7 +2571,7 @@
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>YDR375C</t>
+          <t>YJL063C</t>
         </is>
       </c>
     </row>
@@ -2581,7 +2581,7 @@
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>YJL166W</t>
+          <t>YPL118W</t>
         </is>
       </c>
     </row>
@@ -2591,7 +2591,7 @@
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>YBR251W</t>
+          <t>YDR258C</t>
         </is>
       </c>
     </row>
@@ -2601,7 +2601,7 @@
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>YMR157C</t>
+          <t>YLR203C</t>
         </is>
       </c>
     </row>
@@ -2611,7 +2611,7 @@
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>YGR165W</t>
+          <t>YJL104W</t>
         </is>
       </c>
     </row>
@@ -2621,7 +2621,7 @@
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>YOR266W</t>
+          <t>YML081C-A</t>
         </is>
       </c>
     </row>
@@ -2631,7 +2631,7 @@
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>YMR177W</t>
+          <t>YMR023C</t>
         </is>
       </c>
     </row>
@@ -2641,7 +2641,7 @@
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>YJL133W</t>
+          <t>YJL045W</t>
         </is>
       </c>
     </row>
@@ -2651,7 +2651,7 @@
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>YGL064C</t>
+          <t>YJR003C</t>
         </is>
       </c>
     </row>
@@ -2661,7 +2661,7 @@
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>YEL006W</t>
+          <t>YBR003W</t>
         </is>
       </c>
     </row>
@@ -2671,7 +2671,7 @@
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>YDR065W</t>
+          <t>YCL044C</t>
         </is>
       </c>
     </row>
@@ -2681,7 +2681,7 @@
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>YOR305W</t>
+          <t>YDR322W</t>
         </is>
       </c>
     </row>
@@ -2691,7 +2691,7 @@
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>YMR302C</t>
+          <t>YMR193W</t>
         </is>
       </c>
     </row>
@@ -2701,7 +2701,7 @@
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>YDL119C</t>
+          <t>YNR017W</t>
         </is>
       </c>
     </row>
@@ -2711,7 +2711,7 @@
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>YPL063W</t>
+          <t>YKL011C</t>
         </is>
       </c>
     </row>
@@ -2721,7 +2721,7 @@
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>YMR003W</t>
+          <t>YCR010C</t>
         </is>
       </c>
     </row>
@@ -2731,7 +2731,7 @@
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>YKL056C</t>
+          <t>YPL270W</t>
         </is>
       </c>
     </row>
@@ -2741,7 +2741,7 @@
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>YLR139C</t>
+          <t>YJL166W</t>
         </is>
       </c>
     </row>
@@ -2751,7 +2751,7 @@
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>YMR301C</t>
+          <t>YOR222W</t>
         </is>
       </c>
     </row>
@@ -2761,7 +2761,7 @@
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>YHR135C</t>
+          <t>YLR290C</t>
         </is>
       </c>
     </row>
@@ -2771,7 +2771,7 @@
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>YPL222W</t>
+          <t>YMR301C</t>
         </is>
       </c>
     </row>
@@ -2781,7 +2781,7 @@
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>YGR110W</t>
+          <t>YEL024W</t>
         </is>
       </c>
     </row>
@@ -2791,7 +2791,7 @@
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>YGR062C</t>
+          <t>Q0275</t>
         </is>
       </c>
     </row>
@@ -2801,7 +2801,7 @@
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>YOR211C</t>
+          <t>YPL005W</t>
         </is>
       </c>
     </row>
@@ -2811,7 +2811,7 @@
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>YDR377W</t>
+          <t>YLR084C</t>
         </is>
       </c>
     </row>
@@ -2821,7 +2821,7 @@
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>YLR090W</t>
+          <t>YFL016C</t>
         </is>
       </c>
     </row>
@@ -2831,7 +2831,7 @@
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>YDR236C</t>
+          <t>YKL162C</t>
         </is>
       </c>
     </row>
@@ -2841,7 +2841,7 @@
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>YGR235C</t>
+          <t>YJL054W</t>
         </is>
       </c>
     </row>
@@ -2851,7 +2851,7 @@
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>YPL168W</t>
+          <t>YOR147W</t>
         </is>
       </c>
     </row>
@@ -2861,7 +2861,7 @@
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>YOR297C</t>
+          <t>YDR282C</t>
         </is>
       </c>
     </row>
@@ -2871,7 +2871,7 @@
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>Q0070</t>
+          <t>YDR061W</t>
         </is>
       </c>
     </row>
@@ -2881,7 +2881,7 @@
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>YKL055C</t>
+          <t>YPR149W</t>
         </is>
       </c>
     </row>
@@ -2891,7 +2891,7 @@
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>YPL005W</t>
+          <t>YGR193C</t>
         </is>
       </c>
     </row>
@@ -2911,7 +2911,7 @@
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>YJR003C</t>
+          <t>Q0130</t>
         </is>
       </c>
     </row>
@@ -2921,7 +2921,7 @@
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>YJL023C</t>
+          <t>YDL027C</t>
         </is>
       </c>
     </row>
@@ -2931,7 +2931,7 @@
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>YCR004C</t>
+          <t>YKL208W</t>
         </is>
       </c>
     </row>
@@ -2941,7 +2941,7 @@
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>YDR033W</t>
+          <t>YDR377W</t>
         </is>
       </c>
     </row>
@@ -2951,7 +2951,7 @@
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>YER058W</t>
+          <t>YMR097C</t>
         </is>
       </c>
     </row>
@@ -2961,7 +2961,7 @@
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>YGR174C</t>
+          <t>YDR079W</t>
         </is>
       </c>
     </row>
@@ -2971,7 +2971,7 @@
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>YMR241W</t>
+          <t>YPR020W</t>
         </is>
       </c>
     </row>
@@ -2981,7 +2981,7 @@
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>YIL006W</t>
+          <t>YBR047W</t>
         </is>
       </c>
     </row>
@@ -2991,7 +2991,7 @@
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>Q0085</t>
+          <t>YKL003C</t>
         </is>
       </c>
     </row>
@@ -3001,7 +3001,7 @@
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>YLR204W</t>
+          <t>YJL180C</t>
         </is>
       </c>
     </row>
@@ -3011,7 +3011,7 @@
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>YLR008C</t>
+          <t>YGR257C</t>
         </is>
       </c>
     </row>
@@ -3021,7 +3021,7 @@
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>YNR017W</t>
+          <t>YJL062W-A</t>
         </is>
       </c>
     </row>
@@ -3031,7 +3031,7 @@
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>YEL059C-A</t>
+          <t>YBR227C</t>
         </is>
       </c>
     </row>
@@ -3041,7 +3041,7 @@
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>YLR091W</t>
+          <t>YKL195W</t>
         </is>
       </c>
     </row>
@@ -3051,7 +3051,7 @@
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>YML129C</t>
+          <t>YPR024W</t>
         </is>
       </c>
     </row>
@@ -3061,7 +3061,7 @@
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>YDL036C</t>
+          <t>YDR185C</t>
         </is>
       </c>
     </row>
@@ -3071,7 +3071,7 @@
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>YLR439W</t>
+          <t>YBR251W</t>
         </is>
       </c>
     </row>
@@ -3081,7 +3081,7 @@
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>YGL226W</t>
+          <t>YHR168W</t>
         </is>
       </c>
     </row>
@@ -3091,7 +3091,7 @@
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>YNL256W</t>
+          <t>Q0050</t>
         </is>
       </c>
     </row>
@@ -3101,7 +3101,7 @@
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>YOR350C</t>
+          <t>YOL053W</t>
         </is>
       </c>
     </row>
@@ -3111,7 +3111,7 @@
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>YGL191W</t>
+          <t>YGL236C</t>
         </is>
       </c>
     </row>
@@ -3121,7 +3121,7 @@
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>YER166W</t>
+          <t>YBL038W</t>
         </is>
       </c>
     </row>
@@ -3131,7 +3131,7 @@
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>YHR100C</t>
+          <t>YOR201C</t>
         </is>
       </c>
     </row>
@@ -3141,7 +3141,7 @@
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>YMR307W</t>
+          <t>YFR011C</t>
         </is>
       </c>
     </row>
@@ -3151,7 +3151,7 @@
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>YML120C</t>
+          <t>YPL099C</t>
         </is>
       </c>
     </row>
@@ -3161,7 +3161,7 @@
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>YPL078C</t>
+          <t>YNL185C</t>
         </is>
       </c>
     </row>
@@ -3171,7 +3171,7 @@
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>YKR087C</t>
+          <t>YHR001W-A</t>
         </is>
       </c>
     </row>
@@ -3181,7 +3181,7 @@
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>YLR342W</t>
+          <t>YER080W</t>
         </is>
       </c>
     </row>
@@ -3191,7 +3191,7 @@
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>YPR020W</t>
+          <t>YER017C</t>
         </is>
       </c>
     </row>
@@ -3201,7 +3201,7 @@
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>YPL099C</t>
+          <t>YDL044C</t>
         </is>
       </c>
     </row>
@@ -3211,7 +3211,7 @@
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>YJR045C</t>
+          <t>YFR045W</t>
         </is>
       </c>
     </row>
@@ -3221,7 +3221,7 @@
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>YOL059W</t>
+          <t>YJR077C</t>
         </is>
       </c>
     </row>
@@ -3231,7 +3231,7 @@
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>YMR115W</t>
+          <t>YIR024C</t>
         </is>
       </c>
     </row>
@@ -3241,7 +3241,7 @@
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>YHR162W</t>
+          <t>YEL030W</t>
         </is>
       </c>
     </row>
@@ -3251,7 +3251,7 @@
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>YJL003W</t>
+          <t>YHR005C-A</t>
         </is>
       </c>
     </row>
@@ -3261,7 +3261,7 @@
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>YPR166C</t>
+          <t>YML052W</t>
         </is>
       </c>
     </row>
@@ -3271,7 +3271,7 @@
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>YCL009C</t>
+          <t>YBR262C</t>
         </is>
       </c>
     </row>
@@ -3281,7 +3281,7 @@
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>YNL125C</t>
+          <t>YLR439W</t>
         </is>
       </c>
     </row>
@@ -3291,7 +3291,7 @@
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>YGR033C</t>
+          <t>YPL029W</t>
         </is>
       </c>
     </row>
@@ -3301,7 +3301,7 @@
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>YMR166C</t>
+          <t>YGR033C</t>
         </is>
       </c>
     </row>
@@ -3311,7 +3311,7 @@
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>YDR350C</t>
+          <t>YPL224C</t>
         </is>
       </c>
     </row>
@@ -3321,7 +3321,7 @@
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>YJR077C</t>
+          <t>YDR405W</t>
         </is>
       </c>
     </row>
@@ -3331,7 +3331,7 @@
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>YOR222W</t>
+          <t>YNL098C</t>
         </is>
       </c>
     </row>
@@ -3341,7 +3341,7 @@
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>YLR251W</t>
+          <t>YOR020W-A</t>
         </is>
       </c>
     </row>
@@ -3351,7 +3351,7 @@
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>YJL180C</t>
+          <t>YDR462W</t>
         </is>
       </c>
     </row>
@@ -3361,7 +3361,7 @@
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>YIL042C</t>
+          <t>YJR100C</t>
         </is>
       </c>
     </row>
@@ -3371,7 +3371,7 @@
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>YLL041C</t>
+          <t>YGR084C</t>
         </is>
       </c>
     </row>
@@ -3381,7 +3381,7 @@
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>YLR289W</t>
+          <t>YEL059C-A</t>
         </is>
       </c>
     </row>
@@ -3391,7 +3391,7 @@
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>YPL172C</t>
+          <t>YMR003W</t>
         </is>
       </c>
     </row>
@@ -3401,7 +3401,7 @@
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>YDR462W</t>
+          <t>YDL202W</t>
         </is>
       </c>
     </row>
@@ -3411,7 +3411,7 @@
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>YPL109C</t>
+          <t>YOR334W</t>
         </is>
       </c>
     </row>
@@ -3421,7 +3421,7 @@
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>YHL038C</t>
+          <t>YOR022C</t>
         </is>
       </c>
     </row>
@@ -3431,7 +3431,7 @@
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>YIR021W</t>
+          <t>Q0140</t>
         </is>
       </c>
     </row>
@@ -3441,7 +3441,7 @@
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>YHR194W</t>
+          <t>YPL109C</t>
         </is>
       </c>
     </row>
@@ -3451,7 +3451,7 @@
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>YDR119W-A</t>
+          <t>YOR350C</t>
         </is>
       </c>
     </row>
@@ -3461,7 +3461,7 @@
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>YDR494W</t>
+          <t>YLR164W</t>
         </is>
       </c>
     </row>
@@ -3471,7 +3471,7 @@
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>YBL059W</t>
+          <t>YJL003W</t>
         </is>
       </c>
     </row>
@@ -3481,7 +3481,7 @@
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>YIL077C</t>
+          <t>Q0120</t>
         </is>
       </c>
     </row>
@@ -3491,7 +3491,7 @@
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>YNR040W</t>
+          <t>YML120C</t>
         </is>
       </c>
     </row>
@@ -3501,7 +3501,7 @@
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>YEL024W</t>
+          <t>YJL023C</t>
         </is>
       </c>
     </row>
@@ -3511,7 +3511,7 @@
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>YGR084C</t>
+          <t>YBR091C</t>
         </is>
       </c>
     </row>
@@ -3521,7 +3521,7 @@
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>YPL224C</t>
+          <t>YML025C</t>
         </is>
       </c>
     </row>
@@ -3531,7 +3531,7 @@
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>YEL052W</t>
+          <t>YPR021C</t>
         </is>
       </c>
     </row>
@@ -3541,7 +3541,7 @@
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>YNL252C</t>
+          <t>YMR108W</t>
         </is>
       </c>
     </row>
@@ -3551,7 +3551,7 @@
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>YFR011C</t>
+          <t>YLR201C</t>
         </is>
       </c>
     </row>
@@ -3561,7 +3561,7 @@
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>YPL097W</t>
+          <t>YLR077W</t>
         </is>
       </c>
     </row>
@@ -3571,7 +3571,7 @@
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>YOR176W</t>
+          <t>YDL036C</t>
         </is>
       </c>
     </row>
@@ -3581,7 +3581,7 @@
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>YHR168W</t>
+          <t>YCL057C-A</t>
         </is>
       </c>
     </row>
@@ -3591,7 +3591,7 @@
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>YFR045W</t>
+          <t>YLR395C</t>
         </is>
       </c>
     </row>
@@ -3601,7 +3601,7 @@
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>YJR095W</t>
+          <t>YMR212C</t>
         </is>
       </c>
     </row>
@@ -3611,7 +3611,7 @@
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>YBL022C</t>
+          <t>YER020W</t>
         </is>
       </c>
     </row>
@@ -3621,7 +3621,7 @@
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>YMR023C</t>
+          <t>YGR147C</t>
         </is>
       </c>
     </row>
@@ -3631,7 +3631,7 @@
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>YGL129C</t>
+          <t>YJR095W</t>
         </is>
       </c>
     </row>
@@ -3641,7 +3641,7 @@
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>YJL104W</t>
+          <t>YPR116W</t>
         </is>
       </c>
     </row>
@@ -3651,7 +3651,7 @@
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>YDR298C</t>
+          <t>YBR039W</t>
         </is>
       </c>
     </row>
@@ -3661,7 +3661,7 @@
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>YPR021C</t>
+          <t>YIL022W</t>
         </is>
       </c>
     </row>
@@ -3671,7 +3671,7 @@
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>YOL042W</t>
+          <t>YPL060W</t>
         </is>
       </c>
     </row>
@@ -3681,7 +3681,7 @@
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>YDR258C</t>
+          <t>YMR157C</t>
         </is>
       </c>
     </row>
@@ -3691,7 +3691,7 @@
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>YBR192W</t>
+          <t>YDL085W</t>
         </is>
       </c>
     </row>
@@ -3701,7 +3701,7 @@
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>YGR183C</t>
+          <t>YGR132C</t>
         </is>
       </c>
     </row>
@@ -3711,7 +3711,7 @@
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>YDR041W</t>
+          <t>YBL030C</t>
         </is>
       </c>
     </row>
@@ -3721,7 +3721,7 @@
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>YHR120W</t>
+          <t>YBR085W</t>
         </is>
       </c>
     </row>
@@ -3731,7 +3731,7 @@
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>YNL211C</t>
+          <t>YPL215W</t>
         </is>
       </c>
     </row>
@@ -3741,7 +3741,7 @@
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t>YIR024C</t>
+          <t>Q0070</t>
         </is>
       </c>
     </row>
@@ -3751,7 +3751,7 @@
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>YER077C</t>
+          <t>YKR016W</t>
         </is>
       </c>
     </row>
@@ -3761,7 +3761,7 @@
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>YPL215W</t>
+          <t>YOR017W</t>
         </is>
       </c>
     </row>
@@ -3771,7 +3771,7 @@
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>YDR204W</t>
+          <t>YLR390W</t>
         </is>
       </c>
     </row>
@@ -3781,7 +3781,7 @@
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t>YNR045W</t>
+          <t>YBR084W</t>
         </is>
       </c>
     </row>
@@ -3791,7 +3791,7 @@
       </c>
       <c r="B337" t="inlineStr">
         <is>
-          <t>YDR233C</t>
+          <t>YHR147C</t>
         </is>
       </c>
     </row>
@@ -3801,7 +3801,7 @@
       </c>
       <c r="B338" t="inlineStr">
         <is>
-          <t>YBR054W</t>
+          <t>YAL039C</t>
         </is>
       </c>
     </row>
@@ -3811,7 +3811,7 @@
       </c>
       <c r="B339" t="inlineStr">
         <is>
-          <t>YPR058W</t>
+          <t>YGL064C</t>
         </is>
       </c>
     </row>
@@ -3821,7 +3821,7 @@
       </c>
       <c r="B340" t="inlineStr">
         <is>
-          <t>YPR116W</t>
+          <t>YLR038C</t>
         </is>
       </c>
     </row>
@@ -3831,7 +3831,7 @@
       </c>
       <c r="B341" t="inlineStr">
         <is>
-          <t>YER168C</t>
+          <t>YMR056C</t>
         </is>
       </c>
     </row>
@@ -3841,7 +3841,7 @@
       </c>
       <c r="B342" t="inlineStr">
         <is>
-          <t>YLR038C</t>
+          <t>YBR121C</t>
         </is>
       </c>
     </row>
@@ -3851,7 +3851,7 @@
       </c>
       <c r="B343" t="inlineStr">
         <is>
-          <t>YNR002C</t>
+          <t>YER019W</t>
         </is>
       </c>
     </row>
@@ -3861,7 +3861,7 @@
       </c>
       <c r="B344" t="inlineStr">
         <is>
-          <t>YML030W</t>
+          <t>YMR307W</t>
         </is>
       </c>
     </row>
@@ -3871,7 +3871,7 @@
       </c>
       <c r="B345" t="inlineStr">
         <is>
-          <t>YJL063C</t>
+          <t>YLR059C</t>
         </is>
       </c>
     </row>
@@ -3881,7 +3881,7 @@
       </c>
       <c r="B346" t="inlineStr">
         <is>
-          <t>YKL133C</t>
+          <t>YKL106W</t>
         </is>
       </c>
     </row>
@@ -3891,7 +3891,7 @@
       </c>
       <c r="B347" t="inlineStr">
         <is>
-          <t>YKL162C</t>
+          <t>YOR221C</t>
         </is>
       </c>
     </row>
@@ -3901,7 +3901,7 @@
       </c>
       <c r="B348" t="inlineStr">
         <is>
-          <t>YGL057C</t>
+          <t>YMR158W</t>
         </is>
       </c>
     </row>
@@ -3911,7 +3911,7 @@
       </c>
       <c r="B349" t="inlineStr">
         <is>
-          <t>YGR231C</t>
+          <t>YNL071W</t>
         </is>
       </c>
     </row>
@@ -3921,7 +3921,7 @@
       </c>
       <c r="B350" t="inlineStr">
         <is>
-          <t>YKL155C</t>
+          <t>YDL198C</t>
         </is>
       </c>
     </row>
@@ -3931,7 +3931,7 @@
       </c>
       <c r="B351" t="inlineStr">
         <is>
-          <t>YOR271C</t>
+          <t>YNL315C</t>
         </is>
       </c>
     </row>
@@ -3941,7 +3941,7 @@
       </c>
       <c r="B352" t="inlineStr">
         <is>
-          <t>YPR125W</t>
+          <t>YCR004C</t>
         </is>
       </c>
     </row>
@@ -3951,7 +3951,7 @@
       </c>
       <c r="B353" t="inlineStr">
         <is>
-          <t>YKL187C</t>
+          <t>YBR054W</t>
         </is>
       </c>
     </row>
@@ -3961,7 +3961,7 @@
       </c>
       <c r="B354" t="inlineStr">
         <is>
-          <t>YDL067C</t>
+          <t>YJL147C</t>
         </is>
       </c>
     </row>
@@ -3971,7 +3971,7 @@
       </c>
       <c r="B355" t="inlineStr">
         <is>
-          <t>YDR529C</t>
+          <t>YMR024W</t>
         </is>
       </c>
     </row>
@@ -3981,7 +3981,7 @@
       </c>
       <c r="B356" t="inlineStr">
         <is>
-          <t>YPL231W</t>
+          <t>YHR100C</t>
         </is>
       </c>
     </row>
@@ -3991,7 +3991,7 @@
       </c>
       <c r="B357" t="inlineStr">
         <is>
-          <t>YER153C</t>
+          <t>YMR241W</t>
         </is>
       </c>
     </row>
@@ -4001,7 +4001,7 @@
       </c>
       <c r="B358" t="inlineStr">
         <is>
-          <t>YBL045C</t>
+          <t>YNL328C</t>
         </is>
       </c>
     </row>
@@ -4011,7 +4011,7 @@
       </c>
       <c r="B359" t="inlineStr">
         <is>
-          <t>YNL071W</t>
+          <t>YHR120W</t>
         </is>
       </c>
     </row>
@@ -4021,7 +4021,7 @@
       </c>
       <c r="B360" t="inlineStr">
         <is>
-          <t>YKL113C</t>
+          <t>YNL125C</t>
         </is>
       </c>
     </row>
@@ -4031,7 +4031,7 @@
       </c>
       <c r="B361" t="inlineStr">
         <is>
-          <t>YPR140W</t>
+          <t>YKL120W</t>
         </is>
       </c>
     </row>
@@ -4041,7 +4041,7 @@
       </c>
       <c r="B362" t="inlineStr">
         <is>
-          <t>YJL161W</t>
+          <t>YKL134C</t>
         </is>
       </c>
     </row>
@@ -4051,7 +4051,7 @@
       </c>
       <c r="B363" t="inlineStr">
         <is>
-          <t>YOR130C</t>
+          <t>YMR166C</t>
         </is>
       </c>
     </row>
@@ -4061,7 +4061,7 @@
       </c>
       <c r="B364" t="inlineStr">
         <is>
-          <t>YDR178W</t>
+          <t>YNL005C</t>
         </is>
       </c>
     </row>
@@ -4071,7 +4071,7 @@
       </c>
       <c r="B365" t="inlineStr">
         <is>
-          <t>Q0060</t>
+          <t>YNL306W</t>
         </is>
       </c>
     </row>
@@ -4081,7 +4081,7 @@
       </c>
       <c r="B366" t="inlineStr">
         <is>
-          <t>YKL106W</t>
+          <t>YJR080C</t>
         </is>
       </c>
     </row>
@@ -4091,7 +4091,7 @@
       </c>
       <c r="B367" t="inlineStr">
         <is>
-          <t>YBR262C</t>
+          <t>YGR171C</t>
         </is>
       </c>
     </row>
@@ -4101,7 +4101,7 @@
       </c>
       <c r="B368" t="inlineStr">
         <is>
-          <t>YKR065C</t>
+          <t>YDR236C</t>
         </is>
       </c>
     </row>
@@ -4111,7 +4111,7 @@
       </c>
       <c r="B369" t="inlineStr">
         <is>
-          <t>YCL017C</t>
+          <t>YBL059W</t>
         </is>
       </c>
     </row>
@@ -4121,7 +4121,7 @@
       </c>
       <c r="B370" t="inlineStr">
         <is>
-          <t>YOR022C</t>
+          <t>Q0250</t>
         </is>
       </c>
     </row>
@@ -4131,7 +4131,7 @@
       </c>
       <c r="B371" t="inlineStr">
         <is>
-          <t>YDR381C-A</t>
+          <t>YMR064W</t>
         </is>
       </c>
     </row>
@@ -4141,7 +4141,7 @@
       </c>
       <c r="B372" t="inlineStr">
         <is>
-          <t>YMR256C</t>
+          <t>YLR253W</t>
         </is>
       </c>
     </row>
@@ -4151,7 +4151,7 @@
       </c>
       <c r="B373" t="inlineStr">
         <is>
-          <t>Q0045</t>
+          <t>YKL016C</t>
         </is>
       </c>
     </row>
@@ -4161,7 +4161,7 @@
       </c>
       <c r="B374" t="inlineStr">
         <is>
-          <t>YER020W</t>
+          <t>YLR251W</t>
         </is>
       </c>
     </row>
@@ -4171,7 +4171,7 @@
       </c>
       <c r="B375" t="inlineStr">
         <is>
-          <t>YDR194C</t>
+          <t>YDR381C-A</t>
         </is>
       </c>
     </row>
@@ -4181,7 +4181,7 @@
       </c>
       <c r="B376" t="inlineStr">
         <is>
-          <t>YJL209W</t>
+          <t>YOL008W</t>
         </is>
       </c>
     </row>
@@ -4191,7 +4191,7 @@
       </c>
       <c r="B377" t="inlineStr">
         <is>
-          <t>YER017C</t>
+          <t>YBR185C</t>
         </is>
       </c>
     </row>
@@ -4201,7 +4201,7 @@
       </c>
       <c r="B378" t="inlineStr">
         <is>
-          <t>YIL111W</t>
+          <t>YBR163W</t>
         </is>
       </c>
     </row>
@@ -4211,7 +4211,7 @@
       </c>
       <c r="B379" t="inlineStr">
         <is>
-          <t>YMR089C</t>
+          <t>YJL171C</t>
         </is>
       </c>
     </row>
@@ -4221,7 +4221,7 @@
       </c>
       <c r="B380" t="inlineStr">
         <is>
-          <t>YPR149W</t>
+          <t>YDL164C</t>
         </is>
       </c>
     </row>
@@ -4231,7 +4231,7 @@
       </c>
       <c r="B381" t="inlineStr">
         <is>
-          <t>YIL016W</t>
+          <t>YER125W</t>
         </is>
       </c>
     </row>
@@ -4241,7 +4241,7 @@
       </c>
       <c r="B382" t="inlineStr">
         <is>
-          <t>YAL039C</t>
+          <t>YDR204W</t>
         </is>
       </c>
     </row>
@@ -4251,7 +4251,7 @@
       </c>
       <c r="B383" t="inlineStr">
         <is>
-          <t>YKL217W</t>
+          <t>YJL161W</t>
         </is>
       </c>
     </row>
@@ -4261,7 +4261,7 @@
       </c>
       <c r="B384" t="inlineStr">
         <is>
-          <t>YNL315C</t>
+          <t>YER053C</t>
         </is>
       </c>
     </row>
@@ -4271,7 +4271,7 @@
       </c>
       <c r="B385" t="inlineStr">
         <is>
-          <t>YLR201C</t>
+          <t>YIL105C</t>
         </is>
       </c>
     </row>
@@ -4281,7 +4281,7 @@
       </c>
       <c r="B386" t="inlineStr">
         <is>
-          <t>YKL138C</t>
+          <t>YEL052W</t>
         </is>
       </c>
     </row>
@@ -4291,7 +4291,7 @@
       </c>
       <c r="B387" t="inlineStr">
         <is>
-          <t>Q0140</t>
+          <t>YOR305W</t>
         </is>
       </c>
     </row>
@@ -4301,7 +4301,7 @@
       </c>
       <c r="B388" t="inlineStr">
         <is>
-          <t>YJL171C</t>
+          <t>YDL069C</t>
         </is>
       </c>
     </row>
@@ -4311,7 +4311,7 @@
       </c>
       <c r="B389" t="inlineStr">
         <is>
-          <t>YBR282W</t>
+          <t>YDL183C</t>
         </is>
       </c>
     </row>
@@ -4321,7 +4321,7 @@
       </c>
       <c r="B390" t="inlineStr">
         <is>
-          <t>YML081C-A</t>
+          <t>YPR058W</t>
         </is>
       </c>
     </row>
@@ -4331,7 +4331,7 @@
       </c>
       <c r="B391" t="inlineStr">
         <is>
-          <t>YJL208C</t>
+          <t>YDR529C</t>
         </is>
       </c>
     </row>
@@ -4341,7 +4341,7 @@
       </c>
       <c r="B392" t="inlineStr">
         <is>
-          <t>YMR282C</t>
+          <t>YPR033C</t>
         </is>
       </c>
     </row>
@@ -4351,7 +4351,7 @@
       </c>
       <c r="B393" t="inlineStr">
         <is>
-          <t>YKL134C</t>
+          <t>YOR271C</t>
         </is>
       </c>
     </row>
@@ -4361,7 +4361,7 @@
       </c>
       <c r="B394" t="inlineStr">
         <is>
-          <t>YDR232W</t>
+          <t>YBL013W</t>
         </is>
       </c>
     </row>
@@ -4371,7 +4371,7 @@
       </c>
       <c r="B395" t="inlineStr">
         <is>
-          <t>YHL004W</t>
+          <t>YHR162W</t>
         </is>
       </c>
     </row>
@@ -4381,7 +4381,7 @@
       </c>
       <c r="B396" t="inlineStr">
         <is>
-          <t>YOL096C</t>
+          <t>YGR235C</t>
         </is>
       </c>
     </row>
@@ -4391,7 +4391,7 @@
       </c>
       <c r="B397" t="inlineStr">
         <is>
-          <t>YLR067C</t>
+          <t>YOR330C</t>
         </is>
       </c>
     </row>
@@ -4401,7 +4401,7 @@
       </c>
       <c r="B398" t="inlineStr">
         <is>
-          <t>YOL023W</t>
+          <t>YNL252C</t>
         </is>
       </c>
     </row>
@@ -4411,7 +4411,7 @@
       </c>
       <c r="B399" t="inlineStr">
         <is>
-          <t>YGR257C</t>
+          <t>YDL067C</t>
         </is>
       </c>
     </row>
@@ -4421,7 +4421,7 @@
       </c>
       <c r="B400" t="inlineStr">
         <is>
-          <t>YNL306W</t>
+          <t>YDR384C</t>
         </is>
       </c>
     </row>
@@ -4431,7 +4431,7 @@
       </c>
       <c r="B401" t="inlineStr">
         <is>
-          <t>YHL014C</t>
+          <t>YPL097W</t>
         </is>
       </c>
     </row>
@@ -4441,7 +4441,7 @@
       </c>
       <c r="B402" t="inlineStr">
         <is>
-          <t>YBR037C</t>
+          <t>YDR194C</t>
         </is>
       </c>
     </row>
@@ -4451,7 +4451,7 @@
       </c>
       <c r="B403" t="inlineStr">
         <is>
-          <t>YDR231C</t>
+          <t>YDL142C</t>
         </is>
       </c>
     </row>
@@ -4461,7 +4461,7 @@
       </c>
       <c r="B404" t="inlineStr">
         <is>
-          <t>YKL011C</t>
+          <t>YOR297C</t>
         </is>
       </c>
     </row>
@@ -4471,7 +4471,7 @@
       </c>
       <c r="B405" t="inlineStr">
         <is>
-          <t>YOL077W-A</t>
+          <t>YNL052W</t>
         </is>
       </c>
     </row>
@@ -4481,7 +4481,7 @@
       </c>
       <c r="B406" t="inlineStr">
         <is>
-          <t>YBR085W</t>
+          <t>YGR174C</t>
         </is>
       </c>
     </row>
@@ -4491,7 +4491,7 @@
       </c>
       <c r="B407" t="inlineStr">
         <is>
-          <t>YER080W</t>
+          <t>YML129C</t>
         </is>
       </c>
     </row>
@@ -4501,7 +4501,7 @@
       </c>
       <c r="B408" t="inlineStr">
         <is>
-          <t>YPR134W</t>
+          <t>YKL187C</t>
         </is>
       </c>
     </row>
@@ -4511,7 +4511,7 @@
       </c>
       <c r="B409" t="inlineStr">
         <is>
-          <t>YLR393W</t>
+          <t>YDR322C-A</t>
         </is>
       </c>
     </row>
@@ -4521,7 +4521,7 @@
       </c>
       <c r="B410" t="inlineStr">
         <is>
-          <t>YKL016C</t>
+          <t>YLR289W</t>
         </is>
       </c>
     </row>
@@ -4531,7 +4531,7 @@
       </c>
       <c r="B411" t="inlineStr">
         <is>
-          <t>YBR185C</t>
+          <t>YCL017C</t>
         </is>
       </c>
     </row>
@@ -4541,7 +4541,7 @@
       </c>
       <c r="B412" t="inlineStr">
         <is>
-          <t>YGL080W</t>
+          <t>YGR110W</t>
         </is>
       </c>
     </row>
@@ -4551,7 +4551,7 @@
       </c>
       <c r="B413" t="inlineStr">
         <is>
-          <t>YKL003C</t>
+          <t>YGR096W</t>
         </is>
       </c>
     </row>
@@ -4561,7 +4561,7 @@
       </c>
       <c r="B414" t="inlineStr">
         <is>
-          <t>YMR108W</t>
+          <t>YOL096C</t>
         </is>
       </c>
     </row>
@@ -4571,7 +4571,7 @@
       </c>
       <c r="B415" t="inlineStr">
         <is>
-          <t>YDR116C</t>
+          <t>YKL029C</t>
         </is>
       </c>
     </row>
@@ -4581,7 +4581,7 @@
       </c>
       <c r="B416" t="inlineStr">
         <is>
-          <t>YGL059W</t>
+          <t>YMR115W</t>
         </is>
       </c>
     </row>
@@ -4591,7 +4591,7 @@
       </c>
       <c r="B417" t="inlineStr">
         <is>
-          <t>YIL155C</t>
+          <t>YDR316W</t>
         </is>
       </c>
     </row>
@@ -4601,7 +4601,7 @@
       </c>
       <c r="B418" t="inlineStr">
         <is>
-          <t>Q0110</t>
+          <t>YPL134C</t>
         </is>
       </c>
     </row>
@@ -4611,7 +4611,7 @@
       </c>
       <c r="B419" t="inlineStr">
         <is>
-          <t>YDL222C</t>
+          <t>YIL154C</t>
         </is>
       </c>
     </row>
@@ -4621,7 +4621,7 @@
       </c>
       <c r="B420" t="inlineStr">
         <is>
-          <t>YLR059C</t>
+          <t>YER077C</t>
         </is>
       </c>
     </row>
@@ -4631,7 +4631,7 @@
       </c>
       <c r="B421" t="inlineStr">
         <is>
-          <t>YLR203C</t>
+          <t>YPL222W</t>
         </is>
       </c>
     </row>
@@ -4641,7 +4641,7 @@
       </c>
       <c r="B422" t="inlineStr">
         <is>
-          <t>YBL038W</t>
+          <t>YMR098C</t>
         </is>
       </c>
     </row>
@@ -4651,7 +4651,7 @@
       </c>
       <c r="B423" t="inlineStr">
         <is>
-          <t>YML091C</t>
+          <t>YOL077W-A</t>
         </is>
       </c>
     </row>
@@ -4661,7 +4661,7 @@
       </c>
       <c r="B424" t="inlineStr">
         <is>
-          <t>YER053C</t>
+          <t>YDR197W</t>
         </is>
       </c>
     </row>
@@ -4671,7 +4671,7 @@
       </c>
       <c r="B425" t="inlineStr">
         <is>
-          <t>YKL120W</t>
+          <t>YML110C</t>
         </is>
       </c>
     </row>
@@ -4681,7 +4681,7 @@
       </c>
       <c r="B426" t="inlineStr">
         <is>
-          <t>YKL196C</t>
+          <t>YPL103C</t>
         </is>
       </c>
     </row>
@@ -4691,7 +4691,7 @@
       </c>
       <c r="B427" t="inlineStr">
         <is>
-          <t>YNR041C</t>
+          <t>YBR192W</t>
         </is>
       </c>
     </row>
@@ -4701,7 +4701,7 @@
       </c>
       <c r="B428" t="inlineStr">
         <is>
-          <t>YOR334W</t>
+          <t>YGR046W</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: add new analysis
</commit_message>
<xml_diff>
--- a/data/sce_compartment_curation/mitochondrial_inner_membrane_annotations_manual_v3.xlsx
+++ b/data/sce_compartment_curation/mitochondrial_inner_membrane_annotations_manual_v3.xlsx
@@ -441,7 +441,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>YFR033C</t>
+          <t>YGR183C</t>
         </is>
       </c>
     </row>
@@ -451,7 +451,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>YLR382C</t>
+          <t>YDR058C</t>
         </is>
       </c>
     </row>
@@ -461,7 +461,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>YDL207W</t>
+          <t>YFL016C</t>
         </is>
       </c>
     </row>
@@ -471,7 +471,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>YGL107C</t>
+          <t>YPR125W</t>
         </is>
       </c>
     </row>
@@ -481,7 +481,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>YOR086C</t>
+          <t>YPL118W</t>
         </is>
       </c>
     </row>
@@ -491,7 +491,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>YOR266W</t>
+          <t>YOR017W</t>
         </is>
       </c>
     </row>
@@ -501,7 +501,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>YKL087C</t>
+          <t>YGL064C</t>
         </is>
       </c>
     </row>
@@ -511,7 +511,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>YPL172C</t>
+          <t>YGR243W</t>
         </is>
       </c>
     </row>
@@ -521,7 +521,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>YBR078W</t>
+          <t>YOR354C</t>
         </is>
       </c>
     </row>
@@ -531,7 +531,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>YJR034W</t>
+          <t>YMR023C</t>
         </is>
       </c>
     </row>
@@ -541,7 +541,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>YDR375C</t>
+          <t>YEL052W</t>
         </is>
       </c>
     </row>
@@ -551,7 +551,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>YBR044C</t>
+          <t>YOL023W</t>
         </is>
       </c>
     </row>
@@ -561,7 +561,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>YDL004W</t>
+          <t>YOL053W</t>
         </is>
       </c>
     </row>
@@ -571,7 +571,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>YBL099W</t>
+          <t>YDR405W</t>
         </is>
       </c>
     </row>
@@ -581,7 +581,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>YHL038C</t>
+          <t>YOR211C</t>
         </is>
       </c>
     </row>
@@ -591,7 +591,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>YIL134W</t>
+          <t>YHR011W</t>
         </is>
       </c>
     </row>
@@ -601,7 +601,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>YLR283W</t>
+          <t>YPL109C</t>
         </is>
       </c>
     </row>
@@ -611,7 +611,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>YDR116C</t>
+          <t>YPR061C</t>
         </is>
       </c>
     </row>
@@ -621,7 +621,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>YDR298C</t>
+          <t>YOR020W-A</t>
         </is>
       </c>
     </row>
@@ -631,7 +631,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>YOL059W</t>
+          <t>YPR134W</t>
         </is>
       </c>
     </row>
@@ -641,7 +641,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>YOL042W</t>
+          <t>YER125W</t>
         </is>
       </c>
     </row>
@@ -651,7 +651,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>YDR033W</t>
+          <t>YGR255C</t>
         </is>
       </c>
     </row>
@@ -661,7 +661,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>YPL231W</t>
+          <t>YDL215C</t>
         </is>
       </c>
     </row>
@@ -671,7 +671,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>YML030W</t>
+          <t>YLR390W</t>
         </is>
       </c>
     </row>
@@ -681,7 +681,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>YHR199C</t>
+          <t>YCL044C</t>
         </is>
       </c>
     </row>
@@ -691,7 +691,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>YGR231C</t>
+          <t>YOL095C</t>
         </is>
       </c>
     </row>
@@ -701,7 +701,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>YGL191W</t>
+          <t>YMR098C</t>
         </is>
       </c>
     </row>
@@ -711,7 +711,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>YOR232W</t>
+          <t>YNL122C</t>
         </is>
       </c>
     </row>
@@ -721,7 +721,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>YDR041W</t>
+          <t>YBR024W</t>
         </is>
       </c>
     </row>
@@ -731,7 +731,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>YLR204W</t>
+          <t>YGR147C</t>
         </is>
       </c>
     </row>
@@ -741,7 +741,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>YGL057C</t>
+          <t>YKL056C</t>
         </is>
       </c>
     </row>
@@ -751,7 +751,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>YER166W</t>
+          <t>YKL141W</t>
         </is>
       </c>
     </row>
@@ -761,7 +761,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>YGR222W</t>
+          <t>YKR042W</t>
         </is>
       </c>
     </row>
@@ -771,7 +771,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>YCR046C</t>
+          <t>YEL024W</t>
         </is>
       </c>
     </row>
@@ -781,7 +781,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>YER182W</t>
+          <t>YML128C</t>
         </is>
       </c>
     </row>
@@ -791,7 +791,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>YOL027C</t>
+          <t>YLR290C</t>
         </is>
       </c>
     </row>
@@ -801,7 +801,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>YML128C</t>
+          <t>YMR193W</t>
         </is>
       </c>
     </row>
@@ -811,7 +811,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>YCL009C</t>
+          <t>YMR064W</t>
         </is>
       </c>
     </row>
@@ -821,7 +821,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>YJR101W</t>
+          <t>YLR342W</t>
         </is>
       </c>
     </row>
@@ -831,7 +831,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>YPR125W</t>
+          <t>YBL013W</t>
         </is>
       </c>
     </row>
@@ -841,7 +841,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>YNR002C</t>
+          <t>YIL042C</t>
         </is>
       </c>
     </row>
@@ -851,7 +851,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>YLR239C</t>
+          <t>YOR196C</t>
         </is>
       </c>
     </row>
@@ -861,7 +861,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>YPR191W</t>
+          <t>YKL011C</t>
         </is>
       </c>
     </row>
@@ -871,7 +871,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>YKL138C</t>
+          <t>YOR176W</t>
         </is>
       </c>
     </row>
@@ -881,7 +881,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>YBR037C</t>
+          <t>YOR350C</t>
         </is>
       </c>
     </row>
@@ -891,7 +891,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>YGL080W</t>
+          <t>YHR199C</t>
         </is>
       </c>
     </row>
@@ -901,7 +901,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>YGR112W</t>
+          <t>YJL143W</t>
         </is>
       </c>
     </row>
@@ -911,7 +911,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>YHR135C</t>
+          <t>YLL041C</t>
         </is>
       </c>
     </row>
@@ -921,7 +921,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>YAL054C</t>
+          <t>YGL191W</t>
         </is>
       </c>
     </row>
@@ -931,7 +931,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>YIL006W</t>
+          <t>YEL020W-A</t>
         </is>
       </c>
     </row>
@@ -941,7 +941,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>YMR038C</t>
+          <t>YPR191W</t>
         </is>
       </c>
     </row>
@@ -951,7 +951,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>YGL119W</t>
+          <t>YFR045W</t>
         </is>
       </c>
     </row>
@@ -961,7 +961,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>YPL063W</t>
+          <t>YHR168W</t>
         </is>
       </c>
     </row>
@@ -971,7 +971,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>YHL014C</t>
+          <t>YPL134C</t>
         </is>
       </c>
     </row>
@@ -981,7 +981,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>YLR193C</t>
+          <t>YDR393W</t>
         </is>
       </c>
     </row>
@@ -991,7 +991,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>YMR177W</t>
+          <t>YCR046C</t>
         </is>
       </c>
     </row>
@@ -1001,7 +1001,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>YDR233C</t>
+          <t>YLR204W</t>
         </is>
       </c>
     </row>
@@ -1011,7 +1011,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>YJL102W</t>
+          <t>YDR375C</t>
         </is>
       </c>
     </row>
@@ -1021,7 +1021,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>YER086W</t>
+          <t>YJL208C</t>
         </is>
       </c>
     </row>
@@ -1031,7 +1031,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>YPR061C</t>
+          <t>YDR529C</t>
         </is>
       </c>
     </row>
@@ -1041,7 +1041,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>YOL095C</t>
+          <t>YLR283W</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>YMR302C</t>
+          <t>YMR066W</t>
         </is>
       </c>
     </row>
@@ -1061,7 +1061,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>YLL041C</t>
+          <t>YLR059C</t>
         </is>
       </c>
     </row>
@@ -1071,7 +1071,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>YIL077C</t>
+          <t>YDL164C</t>
         </is>
       </c>
     </row>
@@ -1081,7 +1081,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>YJR121W</t>
+          <t>YMR097C</t>
         </is>
       </c>
     </row>
@@ -1091,7 +1091,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>YKR065C</t>
+          <t>YGL136C</t>
         </is>
       </c>
     </row>
@@ -1101,7 +1101,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>YNR045W</t>
+          <t>YDR377W</t>
         </is>
       </c>
     </row>
@@ -1111,7 +1111,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>YNL100W</t>
+          <t>YDR185C</t>
         </is>
       </c>
     </row>
@@ -1121,7 +1121,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>YGR165W</t>
+          <t>Q0060</t>
         </is>
       </c>
     </row>
@@ -1131,7 +1131,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>YGR236C</t>
+          <t>YMR038C</t>
         </is>
       </c>
     </row>
@@ -1141,7 +1141,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Q0105</t>
+          <t>YDR298C</t>
         </is>
       </c>
     </row>
@@ -1151,7 +1151,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>YNL122C</t>
+          <t>YOR334W</t>
         </is>
       </c>
     </row>
@@ -1161,7 +1161,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>YBR282W</t>
+          <t>YGL226W</t>
         </is>
       </c>
     </row>
@@ -1171,7 +1171,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>YLR312W-A</t>
+          <t>YKL029C</t>
         </is>
       </c>
     </row>
@@ -1181,7 +1181,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>YJL209W</t>
+          <t>YKL148C</t>
         </is>
       </c>
     </row>
@@ -1191,7 +1191,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>YNL211C</t>
+          <t>YEL059C-A</t>
         </is>
       </c>
     </row>
@@ -1201,7 +1201,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>YOR065W</t>
+          <t>YER058W</t>
         </is>
       </c>
     </row>
@@ -1211,7 +1211,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>YJL143W</t>
+          <t>Q0070</t>
         </is>
       </c>
     </row>
@@ -1221,7 +1221,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>YPL168W</t>
+          <t>YPL270W</t>
         </is>
       </c>
     </row>
@@ -1231,7 +1231,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>YGR220C</t>
+          <t>YGL107C</t>
         </is>
       </c>
     </row>
@@ -1241,7 +1241,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>YLR139C</t>
+          <t>YNR041C</t>
         </is>
       </c>
     </row>
@@ -1251,7 +1251,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>YKL141W</t>
+          <t>YIL105C</t>
         </is>
       </c>
     </row>
@@ -1261,7 +1261,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>YKR042W</t>
+          <t>YLR203C</t>
         </is>
       </c>
     </row>
@@ -1271,7 +1271,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>YDR494W</t>
+          <t>YJR034W</t>
         </is>
       </c>
     </row>
@@ -1281,7 +1281,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>YJL133W</t>
+          <t>YOR022C</t>
         </is>
       </c>
     </row>
@@ -1291,7 +1291,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>YKL055C</t>
+          <t>YMR301C</t>
         </is>
       </c>
     </row>
@@ -1301,7 +1301,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>YOR130C</t>
+          <t>YHR002W</t>
         </is>
       </c>
     </row>
@@ -1311,7 +1311,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>YDR376W</t>
+          <t>YKL133C</t>
         </is>
       </c>
     </row>
@@ -1321,7 +1321,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Q0045</t>
+          <t>YOR147W</t>
         </is>
       </c>
     </row>
@@ -1331,7 +1331,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>YER058W</t>
+          <t>YDR065W</t>
         </is>
       </c>
     </row>
@@ -1341,7 +1341,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>YOR100C</t>
+          <t>Q0085</t>
         </is>
       </c>
     </row>
@@ -1351,7 +1351,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Q0110</t>
+          <t>YBL038W</t>
         </is>
       </c>
     </row>
@@ -1361,7 +1361,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>YDR032C</t>
+          <t>YLR067C</t>
         </is>
       </c>
     </row>
@@ -1371,7 +1371,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>YIL111W</t>
+          <t>YGR236C</t>
         </is>
       </c>
     </row>
@@ -1381,7 +1381,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>YIL016W</t>
+          <t>YER182W</t>
         </is>
       </c>
     </row>
@@ -1391,7 +1391,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>YFL046W</t>
+          <t>YPL132W</t>
         </is>
       </c>
     </row>
@@ -1401,7 +1401,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>YKL113C</t>
+          <t>YPR024W</t>
         </is>
       </c>
     </row>
@@ -1411,7 +1411,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>YER154W</t>
+          <t>YLR201C</t>
         </is>
       </c>
     </row>
@@ -1421,7 +1421,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>YDR058C</t>
+          <t>YIL016W</t>
         </is>
       </c>
     </row>
@@ -1431,7 +1431,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>YML091C</t>
+          <t>Q0275</t>
         </is>
       </c>
     </row>
@@ -1441,7 +1441,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>YLR091W</t>
+          <t>YML052W</t>
         </is>
       </c>
     </row>
@@ -1451,7 +1451,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>YHR002W</t>
+          <t>YBL045C</t>
         </is>
       </c>
     </row>
@@ -1461,7 +1461,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>YHR198C</t>
+          <t>YLR139C</t>
         </is>
       </c>
     </row>
@@ -1471,7 +1471,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>YPL132W</t>
+          <t>YMR177W</t>
         </is>
       </c>
     </row>
@@ -1481,7 +1481,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>YBL022C</t>
+          <t>YLR393W</t>
         </is>
       </c>
     </row>
@@ -1491,7 +1491,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>YPL271W</t>
+          <t>YBR044C</t>
         </is>
       </c>
     </row>
@@ -1501,7 +1501,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>YGL226W</t>
+          <t>YIL134W</t>
         </is>
       </c>
     </row>
@@ -1511,7 +1511,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>YOR176W</t>
+          <t>YDL183C</t>
         </is>
       </c>
     </row>
@@ -1521,7 +1521,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>YDR232W</t>
+          <t>YMR089C</t>
         </is>
       </c>
     </row>
@@ -1531,7 +1531,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>YNR041C</t>
+          <t>YJL104W</t>
         </is>
       </c>
     </row>
@@ -1541,7 +1541,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>YKR087C</t>
+          <t>YDR231C</t>
         </is>
       </c>
     </row>
@@ -1551,7 +1551,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>YDR178W</t>
+          <t>YBR291C</t>
         </is>
       </c>
     </row>
@@ -1561,7 +1561,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>YNL177C</t>
+          <t>YNL005C</t>
         </is>
       </c>
     </row>
@@ -1571,7 +1571,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>YKL170W</t>
+          <t>YOR356W</t>
         </is>
       </c>
     </row>
@@ -1581,7 +1581,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>YBR024W</t>
+          <t>YKL087C</t>
         </is>
       </c>
     </row>
@@ -1591,7 +1591,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>YGL136C</t>
+          <t>YDR079W</t>
         </is>
       </c>
     </row>
@@ -1601,7 +1601,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>YBL095W</t>
+          <t>YNL252C</t>
         </is>
       </c>
     </row>
@@ -1611,7 +1611,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>YNL256W</t>
+          <t>YBR078W</t>
         </is>
       </c>
     </row>
@@ -1621,7 +1621,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>YLR295C</t>
+          <t>YPL231W</t>
         </is>
       </c>
     </row>
@@ -1631,7 +1631,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>YIL155C</t>
+          <t>YBR251W</t>
         </is>
       </c>
     </row>
@@ -1641,7 +1641,7 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>YNL169C</t>
+          <t>YKL195W</t>
         </is>
       </c>
     </row>
@@ -1651,7 +1651,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>YGR255C</t>
+          <t>YGR150C</t>
         </is>
       </c>
     </row>
@@ -1661,7 +1661,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>YDR231C</t>
+          <t>YDR032C</t>
         </is>
       </c>
     </row>
@@ -1671,7 +1671,7 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>YIL042C</t>
+          <t>YCL004W</t>
         </is>
       </c>
     </row>
@@ -1681,7 +1681,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>YOR037W</t>
+          <t>YGR046W</t>
         </is>
       </c>
     </row>
@@ -1691,7 +1691,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>YPR011C</t>
+          <t>YPR058W</t>
         </is>
       </c>
     </row>
@@ -1701,7 +1701,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>YNL009W</t>
+          <t>YPL078C</t>
         </is>
       </c>
     </row>
@@ -1711,7 +1711,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>YLR067C</t>
+          <t>YPL029W</t>
         </is>
       </c>
     </row>
@@ -1721,7 +1721,7 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>YHR194W</t>
+          <t>YIL087C</t>
         </is>
       </c>
     </row>
@@ -1731,7 +1731,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>YHR011W</t>
+          <t>YBR282W</t>
         </is>
       </c>
     </row>
@@ -1741,7 +1741,7 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>YER069W</t>
+          <t>YBR163W</t>
         </is>
       </c>
     </row>
@@ -1751,7 +1751,7 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>YDR065W</t>
+          <t>YCL017C</t>
         </is>
       </c>
     </row>
@@ -1761,7 +1761,7 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>YKL133C</t>
+          <t>YNL003C</t>
         </is>
       </c>
     </row>
@@ -1771,7 +1771,7 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>YJL208C</t>
+          <t>YKL106W</t>
         </is>
       </c>
     </row>
@@ -1781,7 +1781,7 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>YKL056C</t>
+          <t>YLR077W</t>
         </is>
       </c>
     </row>
@@ -1791,7 +1791,7 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>Q0160</t>
+          <t>YKR016W</t>
         </is>
       </c>
     </row>
@@ -1801,7 +1801,7 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>YKL148C</t>
+          <t>YDR116C</t>
         </is>
       </c>
     </row>
@@ -1811,7 +1811,7 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>YIL157C</t>
+          <t>YAL054C</t>
         </is>
       </c>
     </row>
@@ -1821,7 +1821,7 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>YER141W</t>
+          <t>YER069W</t>
         </is>
       </c>
     </row>
@@ -1831,7 +1831,7 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>YGR101W</t>
+          <t>YNL137C</t>
         </is>
       </c>
     </row>
@@ -1841,7 +1841,7 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>YER170W</t>
+          <t>YOL042W</t>
         </is>
       </c>
     </row>
@@ -1851,7 +1851,7 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>YKR052C</t>
+          <t>YCL009C</t>
         </is>
       </c>
     </row>
@@ -1861,7 +1861,7 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>YDL174C</t>
+          <t>YNR040W</t>
         </is>
       </c>
     </row>
@@ -1871,7 +1871,7 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>YJR045C</t>
+          <t>YOR271C</t>
         </is>
       </c>
     </row>
@@ -1881,7 +1881,7 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>YLR188W</t>
+          <t>YDL044C</t>
         </is>
       </c>
     </row>
@@ -1891,7 +1891,7 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>YIL087C</t>
+          <t>YLR253W</t>
         </is>
       </c>
     </row>
@@ -1901,7 +1901,7 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>Q0060</t>
+          <t>YJR101W</t>
         </is>
       </c>
     </row>
@@ -1911,7 +1911,7 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>YER168C</t>
+          <t>YGR174C</t>
         </is>
       </c>
     </row>
@@ -1921,7 +1921,7 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>YPL078C</t>
+          <t>YEL006W</t>
         </is>
       </c>
     </row>
@@ -1931,7 +1931,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>YGR243W</t>
+          <t>YER017C</t>
         </is>
       </c>
     </row>
@@ -1941,7 +1941,7 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>YNR018W</t>
+          <t>YDR322W</t>
         </is>
       </c>
     </row>
@@ -1951,7 +1951,7 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>YDL222C</t>
+          <t>YER183C</t>
         </is>
       </c>
     </row>
@@ -1961,7 +1961,7 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>YGR116W</t>
+          <t>YJL209W</t>
         </is>
       </c>
     </row>
@@ -1971,7 +1971,7 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>YOR211C</t>
+          <t>YOL059W</t>
         </is>
       </c>
     </row>
@@ -1981,7 +1981,7 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>YEL020W-A</t>
+          <t>YOR297C</t>
         </is>
       </c>
     </row>
@@ -1991,7 +1991,7 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>YER153C</t>
+          <t>YBR003W</t>
         </is>
       </c>
     </row>
@@ -2001,7 +2001,7 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>YGR183C</t>
+          <t>YKL170W</t>
         </is>
       </c>
     </row>
@@ -2011,7 +2011,7 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>YHL004W</t>
+          <t>YOR201C</t>
         </is>
       </c>
     </row>
@@ -2021,7 +2021,7 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>YNL003C</t>
+          <t>YBR104W</t>
         </is>
       </c>
     </row>
@@ -2031,7 +2031,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>YLR090W</t>
+          <t>YOR130C</t>
         </is>
       </c>
     </row>
@@ -2041,7 +2041,7 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>YOR196C</t>
+          <t>YPL097W</t>
         </is>
       </c>
     </row>
@@ -2051,7 +2051,7 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>YDL217C</t>
+          <t>YDL085W</t>
         </is>
       </c>
     </row>
@@ -2061,7 +2061,7 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>YEL006W</t>
+          <t>YER141W</t>
         </is>
       </c>
     </row>
@@ -2071,7 +2071,7 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>Q0065</t>
+          <t>YMR228W</t>
         </is>
       </c>
     </row>
@@ -2081,7 +2081,7 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>Q0080</t>
+          <t>YDR462W</t>
         </is>
       </c>
     </row>
@@ -2091,7 +2091,7 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>YOR354C</t>
+          <t>YKL217W</t>
         </is>
       </c>
     </row>
@@ -2101,7 +2101,7 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>YGL129C</t>
+          <t>YGR171C</t>
         </is>
       </c>
     </row>
@@ -2111,7 +2111,7 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>YLR393W</t>
+          <t>YGR101W</t>
         </is>
       </c>
     </row>
@@ -2121,7 +2121,7 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>YGR150C</t>
+          <t>YDR350C</t>
         </is>
       </c>
     </row>
@@ -2131,7 +2131,7 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>YLR342W</t>
+          <t>YHL038C</t>
         </is>
       </c>
     </row>
@@ -2141,7 +2141,7 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>YOR356W</t>
+          <t>YDL004W</t>
         </is>
       </c>
     </row>
@@ -2151,7 +2151,7 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>YMR257C</t>
+          <t>YER053C</t>
         </is>
       </c>
     </row>
@@ -2161,7 +2161,7 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>YDR237W</t>
+          <t>YMR257C</t>
         </is>
       </c>
     </row>
@@ -2171,7 +2171,7 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>YMR089C</t>
+          <t>YLR251W</t>
         </is>
       </c>
     </row>
@@ -2181,7 +2181,7 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>YGR062C</t>
+          <t>YER020W</t>
         </is>
       </c>
     </row>
@@ -2191,7 +2191,7 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>Q0085</t>
+          <t>YMR024W</t>
         </is>
       </c>
     </row>
@@ -2201,7 +2201,7 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>YER014W</t>
+          <t>YNL100W</t>
         </is>
       </c>
     </row>
@@ -2211,7 +2211,7 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>YBR104W</t>
+          <t>YLR295C</t>
         </is>
       </c>
     </row>
@@ -2221,7 +2221,7 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>YMR145C</t>
+          <t>YLR008C</t>
         </is>
       </c>
     </row>
@@ -2231,7 +2231,7 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>YPR140W</t>
+          <t>YPR021C</t>
         </is>
       </c>
     </row>
@@ -2241,7 +2241,7 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>YCL004W</t>
+          <t>YLR193C</t>
         </is>
       </c>
     </row>
@@ -2251,7 +2251,7 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>YMR256C</t>
+          <t>YPR140W</t>
         </is>
       </c>
     </row>
@@ -2261,7 +2261,7 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>YGL059W</t>
+          <t>YGL057C</t>
         </is>
       </c>
     </row>
@@ -2271,7 +2271,7 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>YDR119W-A</t>
+          <t>YPL103C</t>
         </is>
       </c>
     </row>
@@ -2281,7 +2281,7 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>YOL023W</t>
+          <t>YGR116W</t>
         </is>
       </c>
     </row>
@@ -2291,7 +2291,7 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>YKL217W</t>
+          <t>YBR037C</t>
         </is>
       </c>
     </row>
@@ -2301,7 +2301,7 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>YLR008C</t>
+          <t>YBR227C</t>
         </is>
       </c>
     </row>
@@ -2311,7 +2311,7 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>YMR066W</t>
+          <t>YJL166W</t>
         </is>
       </c>
     </row>
@@ -2321,7 +2321,7 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>YNR040W</t>
+          <t>YPL215W</t>
         </is>
       </c>
     </row>
@@ -2331,7 +2331,7 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>YMR282C</t>
+          <t>YOR086C</t>
         </is>
       </c>
     </row>
@@ -2341,7 +2341,7 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>YER183C</t>
+          <t>YPR116W</t>
         </is>
       </c>
     </row>
@@ -2351,7 +2351,7 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>YBR291C</t>
+          <t>YER019W</t>
         </is>
       </c>
     </row>
@@ -2361,7 +2361,7 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>YKL155C</t>
+          <t>YGL080W</t>
         </is>
       </c>
     </row>
@@ -2371,7 +2371,7 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>YPR134W</t>
+          <t>YDR384C</t>
         </is>
       </c>
     </row>
@@ -2381,7 +2381,7 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>YDL119C</t>
+          <t>YIL077C</t>
         </is>
       </c>
     </row>
@@ -2391,7 +2391,7 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>YDL215C</t>
+          <t>YLR312W-A</t>
         </is>
       </c>
     </row>
@@ -2401,7 +2401,7 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>YML072C</t>
+          <t>YML081C-A</t>
         </is>
       </c>
     </row>
@@ -2411,7 +2411,7 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>YOR205C</t>
+          <t>YGR112W</t>
         </is>
       </c>
     </row>
@@ -2421,7 +2421,7 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>Q0055</t>
+          <t>YGR231C</t>
         </is>
       </c>
     </row>
@@ -2431,7 +2431,7 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>YKL196C</t>
+          <t>YDR494W</t>
         </is>
       </c>
     </row>
@@ -2441,7 +2441,7 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>YMR228W</t>
+          <t>YBL095W</t>
         </is>
       </c>
     </row>
@@ -2451,7 +2451,7 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>YPR166C</t>
+          <t>Q0050</t>
         </is>
       </c>
     </row>
@@ -2461,7 +2461,7 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>YDR393W</t>
+          <t>YLR038C</t>
         </is>
       </c>
     </row>
@@ -2471,7 +2471,7 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>YLR348C</t>
+          <t>YDL217C</t>
         </is>
       </c>
     </row>
@@ -2481,7 +2481,7 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>YMR150C</t>
+          <t>YGR110W</t>
         </is>
       </c>
     </row>
@@ -2491,7 +2491,7 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>YIR021W</t>
+          <t>YDR033W</t>
         </is>
       </c>
     </row>
@@ -2501,7 +2501,7 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>YFL036W</t>
+          <t>YKL016C</t>
         </is>
       </c>
     </row>
@@ -2511,7 +2511,7 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>YDR347W</t>
+          <t>YPR149W</t>
         </is>
       </c>
     </row>
@@ -2521,7 +2521,7 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>YBL045C</t>
+          <t>YMR108W</t>
         </is>
       </c>
     </row>
@@ -2531,7 +2531,7 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>YOR125C</t>
+          <t>YBR084W</t>
         </is>
       </c>
     </row>
@@ -2541,7 +2541,7 @@
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>YNL137C</t>
+          <t>YLR289W</t>
         </is>
       </c>
     </row>
@@ -2551,7 +2551,7 @@
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>YDR350C</t>
+          <t>YNL315C</t>
         </is>
       </c>
     </row>
@@ -2561,7 +2561,7 @@
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>YPL098C</t>
+          <t>YHR001W-A</t>
         </is>
       </c>
     </row>
@@ -2571,7 +2571,7 @@
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>YJL063C</t>
+          <t>YML072C</t>
         </is>
       </c>
     </row>
@@ -2581,7 +2581,7 @@
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>YPL118W</t>
+          <t>YDL142C</t>
         </is>
       </c>
     </row>
@@ -2591,7 +2591,7 @@
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>YDR258C</t>
+          <t>YER168C</t>
         </is>
       </c>
     </row>
@@ -2601,7 +2601,7 @@
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>YLR203C</t>
+          <t>YHR198C</t>
         </is>
       </c>
     </row>
@@ -2611,7 +2611,7 @@
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>YJL104W</t>
+          <t>YNL306W</t>
         </is>
       </c>
     </row>
@@ -2621,7 +2621,7 @@
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>YML081C-A</t>
+          <t>YDL174C</t>
         </is>
       </c>
     </row>
@@ -2631,7 +2631,7 @@
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>YMR023C</t>
+          <t>YNR045W</t>
         </is>
       </c>
     </row>
@@ -2641,7 +2641,7 @@
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>YJL045W</t>
+          <t>YIL022W</t>
         </is>
       </c>
     </row>
@@ -2651,7 +2651,7 @@
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>YJR003C</t>
+          <t>YDR041W</t>
         </is>
       </c>
     </row>
@@ -2661,7 +2661,7 @@
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>YBR003W</t>
+          <t>YLR084C</t>
         </is>
       </c>
     </row>
@@ -2671,7 +2671,7 @@
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>YCL044C</t>
+          <t>YOL077W-A</t>
         </is>
       </c>
     </row>
@@ -2681,7 +2681,7 @@
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>YDR322W</t>
+          <t>YDR381C-A</t>
         </is>
       </c>
     </row>
@@ -2691,7 +2691,7 @@
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>YMR193W</t>
+          <t>YML120C</t>
         </is>
       </c>
     </row>
@@ -2701,7 +2701,7 @@
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>YNR017W</t>
+          <t>YPR011C</t>
         </is>
       </c>
     </row>
@@ -2711,7 +2711,7 @@
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>YKL011C</t>
+          <t>YHL014C</t>
         </is>
       </c>
     </row>
@@ -2721,7 +2721,7 @@
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>YCR010C</t>
+          <t>YNL211C</t>
         </is>
       </c>
     </row>
@@ -2731,7 +2731,7 @@
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>YPL270W</t>
+          <t>YBL030C</t>
         </is>
       </c>
     </row>
@@ -2741,7 +2741,7 @@
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>YJL166W</t>
+          <t>YKL208W</t>
         </is>
       </c>
     </row>
@@ -2751,7 +2751,7 @@
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>YOR222W</t>
+          <t>YJL054W</t>
         </is>
       </c>
     </row>
@@ -2761,7 +2761,7 @@
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>YLR290C</t>
+          <t>YIL111W</t>
         </is>
       </c>
     </row>
@@ -2771,7 +2771,7 @@
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>YMR301C</t>
+          <t>YML091C</t>
         </is>
       </c>
     </row>
@@ -2781,7 +2781,7 @@
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>YEL024W</t>
+          <t>YPL222W</t>
         </is>
       </c>
     </row>
@@ -2791,7 +2791,7 @@
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>Q0275</t>
+          <t>YBR085W</t>
         </is>
       </c>
     </row>
@@ -2811,7 +2811,7 @@
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>YLR084C</t>
+          <t>YMR166C</t>
         </is>
       </c>
     </row>
@@ -2821,7 +2821,7 @@
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>YFL016C</t>
+          <t>Q0055</t>
         </is>
       </c>
     </row>
@@ -2831,7 +2831,7 @@
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>YKL162C</t>
+          <t>YJL003W</t>
         </is>
       </c>
     </row>
@@ -2841,7 +2841,7 @@
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>YJL054W</t>
+          <t>YDL222C</t>
         </is>
       </c>
     </row>
@@ -2851,7 +2851,7 @@
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>YOR147W</t>
+          <t>YER166W</t>
         </is>
       </c>
     </row>
@@ -2861,7 +2861,7 @@
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>YDR282C</t>
+          <t>YBL022C</t>
         </is>
       </c>
     </row>
@@ -2871,7 +2871,7 @@
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>YDR061W</t>
+          <t>YPR033C</t>
         </is>
       </c>
     </row>
@@ -2881,7 +2881,7 @@
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>YPR149W</t>
+          <t>YDR232W</t>
         </is>
       </c>
     </row>
@@ -2891,7 +2891,7 @@
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>YGR193C</t>
+          <t>YDR322C-A</t>
         </is>
       </c>
     </row>
@@ -2901,7 +2901,7 @@
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>YMR188C</t>
+          <t>YJL045W</t>
         </is>
       </c>
     </row>
@@ -2911,7 +2911,7 @@
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>Q0130</t>
+          <t>YOR305W</t>
         </is>
       </c>
     </row>
@@ -2921,7 +2921,7 @@
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>YDL027C</t>
+          <t>YJL133W</t>
         </is>
       </c>
     </row>
@@ -2931,7 +2931,7 @@
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>YKL208W</t>
+          <t>YOL096C</t>
         </is>
       </c>
     </row>
@@ -2941,7 +2941,7 @@
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>YDR377W</t>
+          <t>YKL155C</t>
         </is>
       </c>
     </row>
@@ -2951,7 +2951,7 @@
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>YMR097C</t>
+          <t>YDL067C</t>
         </is>
       </c>
     </row>
@@ -2961,7 +2961,7 @@
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>YDR079W</t>
+          <t>YBL099W</t>
         </is>
       </c>
     </row>
@@ -2971,7 +2971,7 @@
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>YPR020W</t>
+          <t>YJL102W</t>
         </is>
       </c>
     </row>
@@ -2981,7 +2981,7 @@
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>YBR047W</t>
+          <t>YDR061W</t>
         </is>
       </c>
     </row>
@@ -2991,7 +2991,7 @@
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>YKL003C</t>
+          <t>YER154W</t>
         </is>
       </c>
     </row>
@@ -3001,7 +3001,7 @@
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>YJL180C</t>
+          <t>YDL027C</t>
         </is>
       </c>
     </row>
@@ -3011,7 +3011,7 @@
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>YGR257C</t>
+          <t>YJL062W-A</t>
         </is>
       </c>
     </row>
@@ -3021,7 +3021,7 @@
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>YJL062W-A</t>
+          <t>YDR197W</t>
         </is>
       </c>
     </row>
@@ -3031,7 +3031,7 @@
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>YBR227C</t>
+          <t>YBR121C</t>
         </is>
       </c>
     </row>
@@ -3041,7 +3041,7 @@
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>YKL195W</t>
+          <t>YGR257C</t>
         </is>
       </c>
     </row>
@@ -3051,7 +3051,7 @@
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>YPR024W</t>
+          <t>YFR033C</t>
         </is>
       </c>
     </row>
@@ -3061,7 +3061,7 @@
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>YDR185C</t>
+          <t>YKL134C</t>
         </is>
       </c>
     </row>
@@ -3071,7 +3071,7 @@
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>YBR251W</t>
+          <t>YNL125C</t>
         </is>
       </c>
     </row>
@@ -3081,7 +3081,7 @@
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>YHR168W</t>
+          <t>YOR205C</t>
         </is>
       </c>
     </row>
@@ -3091,7 +3091,7 @@
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>Q0050</t>
+          <t>YOR232W</t>
         </is>
       </c>
     </row>
@@ -3101,7 +3101,7 @@
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>YOL053W</t>
+          <t>YPL063W</t>
         </is>
       </c>
     </row>
@@ -3111,7 +3111,7 @@
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>YGL236C</t>
+          <t>YOL027C</t>
         </is>
       </c>
     </row>
@@ -3121,7 +3121,7 @@
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>YBL038W</t>
+          <t>YJR003C</t>
         </is>
       </c>
     </row>
@@ -3131,7 +3131,7 @@
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>YOR201C</t>
+          <t>YLR188W</t>
         </is>
       </c>
     </row>
@@ -3141,7 +3141,7 @@
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>YFR011C</t>
+          <t>YHR135C</t>
         </is>
       </c>
     </row>
@@ -3151,7 +3151,7 @@
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>YPL099C</t>
+          <t>YDR237W</t>
         </is>
       </c>
     </row>
@@ -3161,7 +3161,7 @@
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>YNL185C</t>
+          <t>YGR165W</t>
         </is>
       </c>
     </row>
@@ -3171,7 +3171,7 @@
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>YHR001W-A</t>
+          <t>YLR239C</t>
         </is>
       </c>
     </row>
@@ -3181,7 +3181,7 @@
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>YER080W</t>
+          <t>YCR010C</t>
         </is>
       </c>
     </row>
@@ -3191,7 +3191,7 @@
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>YER017C</t>
+          <t>YGL059W</t>
         </is>
       </c>
     </row>
@@ -3201,7 +3201,7 @@
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>YDL044C</t>
+          <t>YGR033C</t>
         </is>
       </c>
     </row>
@@ -3211,7 +3211,7 @@
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>YFR045W</t>
+          <t>YMR302C</t>
         </is>
       </c>
     </row>
@@ -3221,7 +3221,7 @@
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>YJR077C</t>
+          <t>YNL098C</t>
         </is>
       </c>
     </row>
@@ -3231,7 +3231,7 @@
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>YIR024C</t>
+          <t>YJL063C</t>
         </is>
       </c>
     </row>
@@ -3241,7 +3241,7 @@
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>YEL030W</t>
+          <t>YNL169C</t>
         </is>
       </c>
     </row>
@@ -3251,7 +3251,7 @@
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>YHR005C-A</t>
+          <t>YER086W</t>
         </is>
       </c>
     </row>
@@ -3261,7 +3261,7 @@
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>YML052W</t>
+          <t>YIR021W</t>
         </is>
       </c>
     </row>
@@ -3271,7 +3271,7 @@
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>YBR262C</t>
+          <t>YHR147C</t>
         </is>
       </c>
     </row>
@@ -3281,7 +3281,7 @@
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>YLR439W</t>
+          <t>YDR258C</t>
         </is>
       </c>
     </row>
@@ -3291,7 +3291,7 @@
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>YPL029W</t>
+          <t>YDR376W</t>
         </is>
       </c>
     </row>
@@ -3301,7 +3301,7 @@
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>YGR033C</t>
+          <t>YFL036W</t>
         </is>
       </c>
     </row>
@@ -3311,7 +3311,7 @@
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>YPL224C</t>
+          <t>YNL009W</t>
         </is>
       </c>
     </row>
@@ -3321,7 +3321,7 @@
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>YDR405W</t>
+          <t>YMR307W</t>
         </is>
       </c>
     </row>
@@ -3331,7 +3331,7 @@
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>YNL098C</t>
+          <t>YLR382C</t>
         </is>
       </c>
     </row>
@@ -3341,7 +3341,7 @@
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>YOR020W-A</t>
+          <t>YGL236C</t>
         </is>
       </c>
     </row>
@@ -3351,7 +3351,7 @@
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>YDR462W</t>
+          <t>YGR220C</t>
         </is>
       </c>
     </row>
@@ -3361,7 +3361,7 @@
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>YJR100C</t>
+          <t>YOR330C</t>
         </is>
       </c>
     </row>
@@ -3371,7 +3371,7 @@
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>YGR084C</t>
+          <t>YOR266W</t>
         </is>
       </c>
     </row>
@@ -3381,7 +3381,7 @@
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>YEL059C-A</t>
+          <t>YDR236C</t>
         </is>
       </c>
     </row>
@@ -3391,7 +3391,7 @@
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>YMR003W</t>
+          <t>YJR077C</t>
         </is>
       </c>
     </row>
@@ -3401,7 +3401,7 @@
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>YDL202W</t>
+          <t>YCL057C-A</t>
         </is>
       </c>
     </row>
@@ -3411,7 +3411,7 @@
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>YOR334W</t>
+          <t>YPL098C</t>
         </is>
       </c>
     </row>
@@ -3421,7 +3421,7 @@
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>YOR022C</t>
+          <t>Q0110</t>
         </is>
       </c>
     </row>
@@ -3431,7 +3431,7 @@
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>Q0140</t>
+          <t>YJL161W</t>
         </is>
       </c>
     </row>
@@ -3441,7 +3441,7 @@
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>YPL109C</t>
+          <t>YLR164W</t>
         </is>
       </c>
     </row>
@@ -3451,7 +3451,7 @@
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>YOR350C</t>
+          <t>YOR037W</t>
         </is>
       </c>
     </row>
@@ -3461,7 +3461,7 @@
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>YLR164W</t>
+          <t>YAL039C</t>
         </is>
       </c>
     </row>
@@ -3471,7 +3471,7 @@
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>YJL003W</t>
+          <t>YIL157C</t>
         </is>
       </c>
     </row>
@@ -3481,7 +3481,7 @@
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>Q0120</t>
+          <t>YGR084C</t>
         </is>
       </c>
     </row>
@@ -3491,7 +3491,7 @@
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>YML120C</t>
+          <t>YDL119C</t>
         </is>
       </c>
     </row>
@@ -3501,7 +3501,7 @@
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>YJL023C</t>
+          <t>Q0160</t>
         </is>
       </c>
     </row>
@@ -3511,7 +3511,7 @@
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>YBR091C</t>
+          <t>YKR087C</t>
         </is>
       </c>
     </row>
@@ -3521,7 +3521,7 @@
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>YML025C</t>
+          <t>YMR241W</t>
         </is>
       </c>
     </row>
@@ -3531,7 +3531,7 @@
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>YPR021C</t>
+          <t>YBR192W</t>
         </is>
       </c>
     </row>
@@ -3541,7 +3541,7 @@
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>YMR108W</t>
+          <t>YDR194C</t>
         </is>
       </c>
     </row>
@@ -3551,7 +3551,7 @@
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>YLR201C</t>
+          <t>YGR062C</t>
         </is>
       </c>
     </row>
@@ -3561,7 +3561,7 @@
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>YLR077W</t>
+          <t>YDR282C</t>
         </is>
       </c>
     </row>
@@ -3571,7 +3571,7 @@
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>YDL036C</t>
+          <t>YLR348C</t>
         </is>
       </c>
     </row>
@@ -3581,7 +3581,7 @@
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>YCL057C-A</t>
+          <t>YMR115W</t>
         </is>
       </c>
     </row>
@@ -3591,7 +3591,7 @@
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>YLR395C</t>
+          <t>YNL177C</t>
         </is>
       </c>
     </row>
@@ -3601,7 +3601,7 @@
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>YMR212C</t>
+          <t>YHR162W</t>
         </is>
       </c>
     </row>
@@ -3611,7 +3611,7 @@
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>YER020W</t>
+          <t>YDL036C</t>
         </is>
       </c>
     </row>
@@ -3621,7 +3621,7 @@
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>YGR147C</t>
+          <t>YDL207W</t>
         </is>
       </c>
     </row>
@@ -3631,7 +3631,7 @@
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>YJR095W</t>
+          <t>YBR185C</t>
         </is>
       </c>
     </row>
@@ -3641,7 +3641,7 @@
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>YPR116W</t>
+          <t>YIR024C</t>
         </is>
       </c>
     </row>
@@ -3651,7 +3651,7 @@
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>YBR039W</t>
+          <t>YML025C</t>
         </is>
       </c>
     </row>
@@ -3661,7 +3661,7 @@
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>YIL022W</t>
+          <t>Q0105</t>
         </is>
       </c>
     </row>
@@ -3671,7 +3671,7 @@
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>YPL060W</t>
+          <t>YDR316W</t>
         </is>
       </c>
     </row>
@@ -3681,7 +3681,7 @@
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>YMR157C</t>
+          <t>YHR100C</t>
         </is>
       </c>
     </row>
@@ -3691,7 +3691,7 @@
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>YDL085W</t>
+          <t>YNL052W</t>
         </is>
       </c>
     </row>
@@ -3701,7 +3701,7 @@
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>YGR132C</t>
+          <t>YMR282C</t>
         </is>
       </c>
     </row>
@@ -3711,7 +3711,7 @@
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>YBL030C</t>
+          <t>YJL147C</t>
         </is>
       </c>
     </row>
@@ -3721,7 +3721,7 @@
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>YBR085W</t>
+          <t>YMR188C</t>
         </is>
       </c>
     </row>
@@ -3731,7 +3731,7 @@
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>YPL215W</t>
+          <t>YJR100C</t>
         </is>
       </c>
     </row>
@@ -3741,7 +3741,7 @@
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t>Q0070</t>
+          <t>YMR145C</t>
         </is>
       </c>
     </row>
@@ -3751,7 +3751,7 @@
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>YKR016W</t>
+          <t>YLR090W</t>
         </is>
       </c>
     </row>
@@ -3761,7 +3761,7 @@
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>YOR017W</t>
+          <t>Q0130</t>
         </is>
       </c>
     </row>
@@ -3771,7 +3771,7 @@
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>YLR390W</t>
+          <t>YLR439W</t>
         </is>
       </c>
     </row>
@@ -3781,7 +3781,7 @@
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t>YBR084W</t>
+          <t>YML129C</t>
         </is>
       </c>
     </row>
@@ -3791,7 +3791,7 @@
       </c>
       <c r="B337" t="inlineStr">
         <is>
-          <t>YHR147C</t>
+          <t>YER077C</t>
         </is>
       </c>
     </row>
@@ -3801,7 +3801,7 @@
       </c>
       <c r="B338" t="inlineStr">
         <is>
-          <t>YAL039C</t>
+          <t>YFR011C</t>
         </is>
       </c>
     </row>
@@ -3811,7 +3811,7 @@
       </c>
       <c r="B339" t="inlineStr">
         <is>
-          <t>YGL064C</t>
+          <t>YKL138C</t>
         </is>
       </c>
     </row>
@@ -3821,7 +3821,7 @@
       </c>
       <c r="B340" t="inlineStr">
         <is>
-          <t>YLR038C</t>
+          <t>YBR054W</t>
         </is>
       </c>
     </row>
@@ -3831,7 +3831,7 @@
       </c>
       <c r="B341" t="inlineStr">
         <is>
-          <t>YMR056C</t>
+          <t>YER170W</t>
         </is>
       </c>
     </row>
@@ -3841,7 +3841,7 @@
       </c>
       <c r="B342" t="inlineStr">
         <is>
-          <t>YBR121C</t>
+          <t>YPR020W</t>
         </is>
       </c>
     </row>
@@ -3851,7 +3851,7 @@
       </c>
       <c r="B343" t="inlineStr">
         <is>
-          <t>YER019W</t>
+          <t>YCR004C</t>
         </is>
       </c>
     </row>
@@ -3861,7 +3861,7 @@
       </c>
       <c r="B344" t="inlineStr">
         <is>
-          <t>YMR307W</t>
+          <t>YGR193C</t>
         </is>
       </c>
     </row>
@@ -3871,7 +3871,7 @@
       </c>
       <c r="B345" t="inlineStr">
         <is>
-          <t>YLR059C</t>
+          <t>YMR157C</t>
         </is>
       </c>
     </row>
@@ -3881,7 +3881,7 @@
       </c>
       <c r="B346" t="inlineStr">
         <is>
-          <t>YKL106W</t>
+          <t>Q0250</t>
         </is>
       </c>
     </row>
@@ -3891,7 +3891,7 @@
       </c>
       <c r="B347" t="inlineStr">
         <is>
-          <t>YOR221C</t>
+          <t>YKR052C</t>
         </is>
       </c>
     </row>
@@ -3901,7 +3901,7 @@
       </c>
       <c r="B348" t="inlineStr">
         <is>
-          <t>YMR158W</t>
+          <t>YOR125C</t>
         </is>
       </c>
     </row>
@@ -3911,7 +3911,7 @@
       </c>
       <c r="B349" t="inlineStr">
         <is>
-          <t>YNL071W</t>
+          <t>YOR221C</t>
         </is>
       </c>
     </row>
@@ -3921,7 +3921,7 @@
       </c>
       <c r="B350" t="inlineStr">
         <is>
-          <t>YDL198C</t>
+          <t>YHR120W</t>
         </is>
       </c>
     </row>
@@ -3931,7 +3931,7 @@
       </c>
       <c r="B351" t="inlineStr">
         <is>
-          <t>YNL315C</t>
+          <t>YDL069C</t>
         </is>
       </c>
     </row>
@@ -3941,7 +3941,7 @@
       </c>
       <c r="B352" t="inlineStr">
         <is>
-          <t>YCR004C</t>
+          <t>YPL168W</t>
         </is>
       </c>
     </row>
@@ -3951,7 +3951,7 @@
       </c>
       <c r="B353" t="inlineStr">
         <is>
-          <t>YBR054W</t>
+          <t>YMR056C</t>
         </is>
       </c>
     </row>
@@ -3961,7 +3961,7 @@
       </c>
       <c r="B354" t="inlineStr">
         <is>
-          <t>YJL147C</t>
+          <t>YIL155C</t>
         </is>
       </c>
     </row>
@@ -3971,7 +3971,7 @@
       </c>
       <c r="B355" t="inlineStr">
         <is>
-          <t>YMR024W</t>
+          <t>YHR005C-A</t>
         </is>
       </c>
     </row>
@@ -3981,7 +3981,7 @@
       </c>
       <c r="B356" t="inlineStr">
         <is>
-          <t>YHR100C</t>
+          <t>YER080W</t>
         </is>
       </c>
     </row>
@@ -3991,7 +3991,7 @@
       </c>
       <c r="B357" t="inlineStr">
         <is>
-          <t>YMR241W</t>
+          <t>YBR091C</t>
         </is>
       </c>
     </row>
@@ -4001,7 +4001,7 @@
       </c>
       <c r="B358" t="inlineStr">
         <is>
-          <t>YNL328C</t>
+          <t>YGL119W</t>
         </is>
       </c>
     </row>
@@ -4011,7 +4011,7 @@
       </c>
       <c r="B359" t="inlineStr">
         <is>
-          <t>YHR120W</t>
+          <t>YNL071W</t>
         </is>
       </c>
     </row>
@@ -4021,7 +4021,7 @@
       </c>
       <c r="B360" t="inlineStr">
         <is>
-          <t>YNL125C</t>
+          <t>YPL099C</t>
         </is>
       </c>
     </row>
@@ -4031,7 +4031,7 @@
       </c>
       <c r="B361" t="inlineStr">
         <is>
-          <t>YKL120W</t>
+          <t>YNR018W</t>
         </is>
       </c>
     </row>
@@ -4041,7 +4041,7 @@
       </c>
       <c r="B362" t="inlineStr">
         <is>
-          <t>YKL134C</t>
+          <t>YKL162C</t>
         </is>
       </c>
     </row>
@@ -4051,7 +4051,7 @@
       </c>
       <c r="B363" t="inlineStr">
         <is>
-          <t>YMR166C</t>
+          <t>YKL187C</t>
         </is>
       </c>
     </row>
@@ -4061,7 +4061,7 @@
       </c>
       <c r="B364" t="inlineStr">
         <is>
-          <t>YNL005C</t>
+          <t>YML030W</t>
         </is>
       </c>
     </row>
@@ -4071,7 +4071,7 @@
       </c>
       <c r="B365" t="inlineStr">
         <is>
-          <t>YNL306W</t>
+          <t>YMR158W</t>
         </is>
       </c>
     </row>
@@ -4081,7 +4081,7 @@
       </c>
       <c r="B366" t="inlineStr">
         <is>
-          <t>YJR080C</t>
+          <t>YKL196C</t>
         </is>
       </c>
     </row>
@@ -4091,7 +4091,7 @@
       </c>
       <c r="B367" t="inlineStr">
         <is>
-          <t>YGR171C</t>
+          <t>YJL180C</t>
         </is>
       </c>
     </row>
@@ -4101,7 +4101,7 @@
       </c>
       <c r="B368" t="inlineStr">
         <is>
-          <t>YDR236C</t>
+          <t>YJR080C</t>
         </is>
       </c>
     </row>
@@ -4111,7 +4111,7 @@
       </c>
       <c r="B369" t="inlineStr">
         <is>
-          <t>YBL059W</t>
+          <t>YNL328C</t>
         </is>
       </c>
     </row>
@@ -4121,7 +4121,7 @@
       </c>
       <c r="B370" t="inlineStr">
         <is>
-          <t>Q0250</t>
+          <t>YDR204W</t>
         </is>
       </c>
     </row>
@@ -4131,7 +4131,7 @@
       </c>
       <c r="B371" t="inlineStr">
         <is>
-          <t>YMR064W</t>
+          <t>YPL060W</t>
         </is>
       </c>
     </row>
@@ -4141,7 +4141,7 @@
       </c>
       <c r="B372" t="inlineStr">
         <is>
-          <t>YLR253W</t>
+          <t>YMR150C</t>
         </is>
       </c>
     </row>
@@ -4151,7 +4151,7 @@
       </c>
       <c r="B373" t="inlineStr">
         <is>
-          <t>YKL016C</t>
+          <t>YMR256C</t>
         </is>
       </c>
     </row>
@@ -4161,7 +4161,7 @@
       </c>
       <c r="B374" t="inlineStr">
         <is>
-          <t>YLR251W</t>
+          <t>YOL008W</t>
         </is>
       </c>
     </row>
@@ -4171,7 +4171,7 @@
       </c>
       <c r="B375" t="inlineStr">
         <is>
-          <t>YDR381C-A</t>
+          <t>YPR166C</t>
         </is>
       </c>
     </row>
@@ -4181,7 +4181,7 @@
       </c>
       <c r="B376" t="inlineStr">
         <is>
-          <t>YOL008W</t>
+          <t>YBL059W</t>
         </is>
       </c>
     </row>
@@ -4191,7 +4191,7 @@
       </c>
       <c r="B377" t="inlineStr">
         <is>
-          <t>YBR185C</t>
+          <t>YER153C</t>
         </is>
       </c>
     </row>
@@ -4201,7 +4201,7 @@
       </c>
       <c r="B378" t="inlineStr">
         <is>
-          <t>YBR163W</t>
+          <t>YJR095W</t>
         </is>
       </c>
     </row>
@@ -4211,7 +4211,7 @@
       </c>
       <c r="B379" t="inlineStr">
         <is>
-          <t>YJL171C</t>
+          <t>YLR395C</t>
         </is>
       </c>
     </row>
@@ -4221,7 +4221,7 @@
       </c>
       <c r="B380" t="inlineStr">
         <is>
-          <t>YDL164C</t>
+          <t>YDR347W</t>
         </is>
       </c>
     </row>
@@ -4231,7 +4231,7 @@
       </c>
       <c r="B381" t="inlineStr">
         <is>
-          <t>YER125W</t>
+          <t>YKR065C</t>
         </is>
       </c>
     </row>
@@ -4241,7 +4241,7 @@
       </c>
       <c r="B382" t="inlineStr">
         <is>
-          <t>YDR204W</t>
+          <t>YNL185C</t>
         </is>
       </c>
     </row>
@@ -4251,7 +4251,7 @@
       </c>
       <c r="B383" t="inlineStr">
         <is>
-          <t>YJL161W</t>
+          <t>YOR065W</t>
         </is>
       </c>
     </row>
@@ -4261,7 +4261,7 @@
       </c>
       <c r="B384" t="inlineStr">
         <is>
-          <t>YER053C</t>
+          <t>YOR222W</t>
         </is>
       </c>
     </row>
@@ -4271,7 +4271,7 @@
       </c>
       <c r="B385" t="inlineStr">
         <is>
-          <t>YIL105C</t>
+          <t>YMR003W</t>
         </is>
       </c>
     </row>
@@ -4281,7 +4281,7 @@
       </c>
       <c r="B386" t="inlineStr">
         <is>
-          <t>YEL052W</t>
+          <t>YGR096W</t>
         </is>
       </c>
     </row>
@@ -4291,7 +4291,7 @@
       </c>
       <c r="B387" t="inlineStr">
         <is>
-          <t>YOR305W</t>
+          <t>YLR091W</t>
         </is>
       </c>
     </row>
@@ -4301,7 +4301,7 @@
       </c>
       <c r="B388" t="inlineStr">
         <is>
-          <t>YDL069C</t>
+          <t>YGR222W</t>
         </is>
       </c>
     </row>
@@ -4311,7 +4311,7 @@
       </c>
       <c r="B389" t="inlineStr">
         <is>
-          <t>YDL183C</t>
+          <t>YBR047W</t>
         </is>
       </c>
     </row>
@@ -4321,7 +4321,7 @@
       </c>
       <c r="B390" t="inlineStr">
         <is>
-          <t>YPR058W</t>
+          <t>YJR045C</t>
         </is>
       </c>
     </row>
@@ -4331,7 +4331,7 @@
       </c>
       <c r="B391" t="inlineStr">
         <is>
-          <t>YDR529C</t>
+          <t>YEL030W</t>
         </is>
       </c>
     </row>
@@ -4341,7 +4341,7 @@
       </c>
       <c r="B392" t="inlineStr">
         <is>
-          <t>YPR033C</t>
+          <t>Q0140</t>
         </is>
       </c>
     </row>
@@ -4351,7 +4351,7 @@
       </c>
       <c r="B393" t="inlineStr">
         <is>
-          <t>YOR271C</t>
+          <t>YNL256W</t>
         </is>
       </c>
     </row>
@@ -4361,7 +4361,7 @@
       </c>
       <c r="B394" t="inlineStr">
         <is>
-          <t>YBL013W</t>
+          <t>YJL023C</t>
         </is>
       </c>
     </row>
@@ -4371,7 +4371,7 @@
       </c>
       <c r="B395" t="inlineStr">
         <is>
-          <t>YHR162W</t>
+          <t>YDL202W</t>
         </is>
       </c>
     </row>
@@ -4381,7 +4381,7 @@
       </c>
       <c r="B396" t="inlineStr">
         <is>
-          <t>YGR235C</t>
+          <t>YNR002C</t>
         </is>
       </c>
     </row>
@@ -4391,7 +4391,7 @@
       </c>
       <c r="B397" t="inlineStr">
         <is>
-          <t>YOR330C</t>
+          <t>YKL113C</t>
         </is>
       </c>
     </row>
@@ -4401,7 +4401,7 @@
       </c>
       <c r="B398" t="inlineStr">
         <is>
-          <t>YNL252C</t>
+          <t>YIL006W</t>
         </is>
       </c>
     </row>
@@ -4411,7 +4411,7 @@
       </c>
       <c r="B399" t="inlineStr">
         <is>
-          <t>YDL067C</t>
+          <t>Q0080</t>
         </is>
       </c>
     </row>
@@ -4421,7 +4421,7 @@
       </c>
       <c r="B400" t="inlineStr">
         <is>
-          <t>YDR384C</t>
+          <t>YGR235C</t>
         </is>
       </c>
     </row>
@@ -4431,7 +4431,7 @@
       </c>
       <c r="B401" t="inlineStr">
         <is>
-          <t>YPL097W</t>
+          <t>YER014W</t>
         </is>
       </c>
     </row>
@@ -4441,7 +4441,7 @@
       </c>
       <c r="B402" t="inlineStr">
         <is>
-          <t>YDR194C</t>
+          <t>YMR212C</t>
         </is>
       </c>
     </row>
@@ -4451,7 +4451,7 @@
       </c>
       <c r="B403" t="inlineStr">
         <is>
-          <t>YDL142C</t>
+          <t>YPL224C</t>
         </is>
       </c>
     </row>
@@ -4461,7 +4461,7 @@
       </c>
       <c r="B404" t="inlineStr">
         <is>
-          <t>YOR297C</t>
+          <t>YKL120W</t>
         </is>
       </c>
     </row>
@@ -4471,7 +4471,7 @@
       </c>
       <c r="B405" t="inlineStr">
         <is>
-          <t>YNL052W</t>
+          <t>Q0065</t>
         </is>
       </c>
     </row>
@@ -4481,7 +4481,7 @@
       </c>
       <c r="B406" t="inlineStr">
         <is>
-          <t>YGR174C</t>
+          <t>YHL004W</t>
         </is>
       </c>
     </row>
@@ -4491,7 +4491,7 @@
       </c>
       <c r="B407" t="inlineStr">
         <is>
-          <t>YML129C</t>
+          <t>Q0045</t>
         </is>
       </c>
     </row>
@@ -4501,7 +4501,7 @@
       </c>
       <c r="B408" t="inlineStr">
         <is>
-          <t>YKL187C</t>
+          <t>YGR132C</t>
         </is>
       </c>
     </row>
@@ -4511,7 +4511,7 @@
       </c>
       <c r="B409" t="inlineStr">
         <is>
-          <t>YDR322C-A</t>
+          <t>YBR262C</t>
         </is>
       </c>
     </row>
@@ -4521,7 +4521,7 @@
       </c>
       <c r="B410" t="inlineStr">
         <is>
-          <t>YLR289W</t>
+          <t>YDR119W-A</t>
         </is>
       </c>
     </row>
@@ -4531,7 +4531,7 @@
       </c>
       <c r="B411" t="inlineStr">
         <is>
-          <t>YCL017C</t>
+          <t>YDR233C</t>
         </is>
       </c>
     </row>
@@ -4541,7 +4541,7 @@
       </c>
       <c r="B412" t="inlineStr">
         <is>
-          <t>YGR110W</t>
+          <t>YGL129C</t>
         </is>
       </c>
     </row>
@@ -4551,7 +4551,7 @@
       </c>
       <c r="B413" t="inlineStr">
         <is>
-          <t>YGR096W</t>
+          <t>YPL271W</t>
         </is>
       </c>
     </row>
@@ -4561,7 +4561,7 @@
       </c>
       <c r="B414" t="inlineStr">
         <is>
-          <t>YOL096C</t>
+          <t>YHR194W</t>
         </is>
       </c>
     </row>
@@ -4571,7 +4571,7 @@
       </c>
       <c r="B415" t="inlineStr">
         <is>
-          <t>YKL029C</t>
+          <t>YBR039W</t>
         </is>
       </c>
     </row>
@@ -4581,7 +4581,7 @@
       </c>
       <c r="B416" t="inlineStr">
         <is>
-          <t>YMR115W</t>
+          <t>YDR178W</t>
         </is>
       </c>
     </row>
@@ -4591,7 +4591,7 @@
       </c>
       <c r="B417" t="inlineStr">
         <is>
-          <t>YDR316W</t>
+          <t>YNR017W</t>
         </is>
       </c>
     </row>
@@ -4601,7 +4601,7 @@
       </c>
       <c r="B418" t="inlineStr">
         <is>
-          <t>YPL134C</t>
+          <t>Q0120</t>
         </is>
       </c>
     </row>
@@ -4611,7 +4611,7 @@
       </c>
       <c r="B419" t="inlineStr">
         <is>
-          <t>YIL154C</t>
+          <t>YKL003C</t>
         </is>
       </c>
     </row>
@@ -4621,7 +4621,7 @@
       </c>
       <c r="B420" t="inlineStr">
         <is>
-          <t>YER077C</t>
+          <t>YJL171C</t>
         </is>
       </c>
     </row>
@@ -4631,7 +4631,7 @@
       </c>
       <c r="B421" t="inlineStr">
         <is>
-          <t>YPL222W</t>
+          <t>YJR121W</t>
         </is>
       </c>
     </row>
@@ -4641,7 +4641,7 @@
       </c>
       <c r="B422" t="inlineStr">
         <is>
-          <t>YMR098C</t>
+          <t>YIL154C</t>
         </is>
       </c>
     </row>
@@ -4651,7 +4651,7 @@
       </c>
       <c r="B423" t="inlineStr">
         <is>
-          <t>YOL077W-A</t>
+          <t>YML110C</t>
         </is>
       </c>
     </row>
@@ -4661,7 +4661,7 @@
       </c>
       <c r="B424" t="inlineStr">
         <is>
-          <t>YDR197W</t>
+          <t>YFL046W</t>
         </is>
       </c>
     </row>
@@ -4671,7 +4671,7 @@
       </c>
       <c r="B425" t="inlineStr">
         <is>
-          <t>YML110C</t>
+          <t>YKL055C</t>
         </is>
       </c>
     </row>
@@ -4681,7 +4681,7 @@
       </c>
       <c r="B426" t="inlineStr">
         <is>
-          <t>YPL103C</t>
+          <t>YDL198C</t>
         </is>
       </c>
     </row>
@@ -4691,7 +4691,7 @@
       </c>
       <c r="B427" t="inlineStr">
         <is>
-          <t>YBR192W</t>
+          <t>YPL172C</t>
         </is>
       </c>
     </row>
@@ -4701,7 +4701,7 @@
       </c>
       <c r="B428" t="inlineStr">
         <is>
-          <t>YGR046W</t>
+          <t>YOR100C</t>
         </is>
       </c>
     </row>

</xml_diff>